<commit_message>
Complete tail rec feature for mxMany
</commit_message>
<xml_diff>
--- a/tests/ExcelProcesser.Tests/resources/testData.xlsx
+++ b/tests/ExcelProcesser.Tests/resources/testData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBC8E719-3B5E-451A-A66B-41C49B792C07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B2C4D06-6ABA-417A-937F-74412618EEA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="279">
   <si>
     <t>Input</t>
     <phoneticPr fontId="3" type="noConversion"/>
@@ -2376,14 +2376,218 @@
     <xf numFmtId="0" fontId="20" fillId="23" borderId="0" xfId="6" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="20" fillId="23" borderId="0" xfId="8" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="20" fillId="12" borderId="0" xfId="6" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="22" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="6" xfId="3">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="9" xfId="3" applyBorder="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="6" xfId="4">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="9" xfId="4" applyBorder="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="12" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="9" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="9" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="6" xfId="3" applyFont="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="9" xfId="3" applyFont="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="13" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="13" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="13" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="14" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="14" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="7" fontId="23" fillId="14" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="7" fontId="23" fillId="14" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2409,215 +2613,26 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="7" fontId="23" fillId="14" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="7" fontId="23" fillId="14" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="6" xfId="3" applyFont="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="9" xfId="3" applyFont="1" applyBorder="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="13" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="13" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="13" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="14" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="14" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="6" xfId="4">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="9" xfId="4" applyBorder="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="12" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="9" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="9" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="6" xfId="3">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="9" xfId="3" applyBorder="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="8" xfId="3" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2631,40 +2646,25 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="40" xfId="3" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="13" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3328,14 +3328,14 @@
       <c r="C6" t="s">
         <v>155</v>
       </c>
-      <c r="D6" s="119" t="s">
+      <c r="D6" s="117" t="s">
         <v>74</v>
       </c>
-      <c r="E6" s="119"/>
-      <c r="G6" s="119" t="s">
+      <c r="E6" s="117"/>
+      <c r="G6" s="117" t="s">
         <v>75</v>
       </c>
-      <c r="H6" s="119"/>
+      <c r="H6" s="117"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -3413,7 +3413,7 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="117" t="s">
+      <c r="A22" s="118" t="s">
         <v>0</v>
       </c>
       <c r="B22" t="s">
@@ -3421,7 +3421,7 @@
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="117"/>
+      <c r="A23" s="118"/>
       <c r="B23" t="s">
         <v>8</v>
       </c>
@@ -3432,7 +3432,7 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="117" t="s">
+      <c r="A27" s="118" t="s">
         <v>0</v>
       </c>
       <c r="B27" t="s">
@@ -3440,13 +3440,13 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="117"/>
+      <c r="A28" s="118"/>
       <c r="B28" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="117"/>
+      <c r="A29" s="118"/>
       <c r="B29" t="s">
         <v>16</v>
       </c>
@@ -3457,7 +3457,7 @@
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32" s="117" t="s">
+      <c r="A32" s="118" t="s">
         <v>0</v>
       </c>
       <c r="B32" t="s">
@@ -3471,10 +3471,10 @@
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" s="117"/>
+      <c r="A33" s="118"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34" s="117"/>
+      <c r="A34" s="118"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
@@ -3482,7 +3482,7 @@
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37" s="117" t="s">
+      <c r="A37" s="118" t="s">
         <v>0</v>
       </c>
       <c r="B37" t="s">
@@ -3493,13 +3493,13 @@
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A38" s="117"/>
+      <c r="A38" s="118"/>
       <c r="C38" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A39" s="117"/>
+      <c r="A39" s="118"/>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
@@ -3507,7 +3507,7 @@
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A42" s="117" t="s">
+      <c r="A42" s="118" t="s">
         <v>0</v>
       </c>
       <c r="B42" t="s">
@@ -3518,13 +3518,13 @@
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A43" s="117"/>
+      <c r="A43" s="118"/>
       <c r="B43" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A44" s="117"/>
+      <c r="A44" s="118"/>
       <c r="B44" t="s">
         <v>20</v>
       </c>
@@ -3535,7 +3535,7 @@
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A48" s="117" t="s">
+      <c r="A48" s="118" t="s">
         <v>0</v>
       </c>
       <c r="B48" t="s">
@@ -3546,13 +3546,13 @@
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A49" s="117"/>
+      <c r="A49" s="118"/>
       <c r="B49" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A50" s="117"/>
+      <c r="A50" s="118"/>
       <c r="B50" t="s">
         <v>25</v>
       </c>
@@ -3563,7 +3563,7 @@
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A53" s="117" t="s">
+      <c r="A53" s="118" t="s">
         <v>0</v>
       </c>
       <c r="B53" s="114" t="s">
@@ -3575,7 +3575,7 @@
       <c r="E53" s="31"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A54" s="117"/>
+      <c r="A54" s="118"/>
       <c r="B54" s="115" t="s">
         <v>274</v>
       </c>
@@ -3585,7 +3585,7 @@
       <c r="D54" s="31"/>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A55" s="117"/>
+      <c r="A55" s="118"/>
       <c r="B55" s="116" t="s">
         <v>272</v>
       </c>
@@ -3594,7 +3594,7 @@
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A56" s="117"/>
+      <c r="A56" s="118"/>
       <c r="B56" s="116" t="s">
         <v>277</v>
       </c>
@@ -3608,7 +3608,7 @@
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A59" s="117" t="s">
+      <c r="A59" s="118" t="s">
         <v>0</v>
       </c>
       <c r="B59" s="31" t="s">
@@ -3622,7 +3622,7 @@
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A60" s="117"/>
+      <c r="A60" s="118"/>
       <c r="B60" s="35" t="s">
         <v>113</v>
       </c>
@@ -3634,7 +3634,7 @@
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A61" s="117"/>
+      <c r="A61" s="118"/>
       <c r="B61" s="35" t="s">
         <v>114</v>
       </c>
@@ -3643,7 +3643,7 @@
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A62" s="117"/>
+      <c r="A62" s="118"/>
       <c r="B62" s="32" t="s">
         <v>116</v>
       </c>
@@ -3654,7 +3654,7 @@
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A65" s="117" t="s">
+      <c r="A65" s="118" t="s">
         <v>0</v>
       </c>
       <c r="B65" t="s">
@@ -3665,13 +3665,13 @@
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A66" s="117"/>
+      <c r="A66" s="118"/>
       <c r="C66" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A67" s="117"/>
+      <c r="A67" s="118"/>
       <c r="C67" t="s">
         <v>37</v>
       </c>
@@ -3777,7 +3777,7 @@
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A86" s="117" t="s">
+      <c r="A86" s="118" t="s">
         <v>0</v>
       </c>
       <c r="B86" t="s">
@@ -3794,10 +3794,10 @@
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A87" s="117"/>
+      <c r="A87" s="118"/>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A88" s="117"/>
+      <c r="A88" s="118"/>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A92" s="1" t="s">
@@ -3805,7 +3805,7 @@
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A93" s="117" t="s">
+      <c r="A93" s="118" t="s">
         <v>0</v>
       </c>
       <c r="B93" t="s">
@@ -3813,19 +3813,19 @@
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A94" s="117"/>
+      <c r="A94" s="118"/>
       <c r="B94" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A95" s="117"/>
+      <c r="A95" s="118"/>
       <c r="B95" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A96" s="117"/>
+      <c r="A96" s="118"/>
       <c r="B96" t="s">
         <v>58</v>
       </c>
@@ -3836,7 +3836,7 @@
       </c>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A101" s="117" t="s">
+      <c r="A101" s="118" t="s">
         <v>0</v>
       </c>
       <c r="B101" t="s">
@@ -3853,10 +3853,10 @@
       </c>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A102" s="117"/>
+      <c r="A102" s="118"/>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A103" s="117"/>
+      <c r="A103" s="118"/>
     </row>
     <row r="106" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A106" s="1" t="s">
@@ -3864,33 +3864,21 @@
       </c>
     </row>
     <row r="107" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A107" s="118" t="s">
+      <c r="A107" s="119" t="s">
         <v>0</v>
       </c>
-      <c r="B107" t="s">
-        <v>269</v>
-      </c>
-      <c r="D107" t="s">
-        <v>270</v>
-      </c>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A108" s="118"/>
+      <c r="A108" s="119"/>
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A109" s="118"/>
-      <c r="B109">
-        <v>2</v>
-      </c>
+      <c r="A109" s="119"/>
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A110" s="118"/>
-      <c r="D110">
-        <v>3</v>
-      </c>
+      <c r="A110" s="119"/>
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A111" s="118"/>
+      <c r="A111" s="119"/>
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A112" s="113"/>
@@ -3946,7 +3934,7 @@
       </c>
     </row>
     <row r="124" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A124" s="117" t="s">
+      <c r="A124" s="118" t="s">
         <v>0</v>
       </c>
       <c r="B124" t="s">
@@ -3966,10 +3954,10 @@
       </c>
     </row>
     <row r="125" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A125" s="117"/>
+      <c r="A125" s="118"/>
     </row>
     <row r="126" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A126" s="117"/>
+      <c r="A126" s="118"/>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A129" s="1" t="s">
@@ -3977,7 +3965,7 @@
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A130" s="117" t="s">
+      <c r="A130" s="118" t="s">
         <v>0</v>
       </c>
       <c r="B130" t="s">
@@ -3991,10 +3979,10 @@
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A131" s="117"/>
+      <c r="A131" s="118"/>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A132" s="117"/>
+      <c r="A132" s="118"/>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A137" s="1" t="s">
@@ -4002,7 +3990,7 @@
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A138" s="117" t="s">
+      <c r="A138" s="118" t="s">
         <v>0</v>
       </c>
       <c r="B138" t="s">
@@ -4022,10 +4010,10 @@
       </c>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A139" s="117"/>
+      <c r="A139" s="118"/>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A140" s="117"/>
+      <c r="A140" s="118"/>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A143" s="1" t="s">
@@ -4033,7 +4021,7 @@
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A144" s="117" t="s">
+      <c r="A144" s="118" t="s">
         <v>0</v>
       </c>
       <c r="B144" t="s">
@@ -4053,13 +4041,16 @@
       </c>
     </row>
     <row r="145" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A145" s="117"/>
+      <c r="A145" s="118"/>
     </row>
     <row r="146" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A146" s="117"/>
+      <c r="A146" s="118"/>
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="A130:A132"/>
+    <mergeCell ref="A144:A146"/>
+    <mergeCell ref="A53:A56"/>
     <mergeCell ref="D6:E6"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="A124:A126"/>
@@ -4076,9 +4067,6 @@
     <mergeCell ref="A32:A34"/>
     <mergeCell ref="A107:A111"/>
     <mergeCell ref="A59:A62"/>
-    <mergeCell ref="A130:A132"/>
-    <mergeCell ref="A144:A146"/>
-    <mergeCell ref="A53:A56"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4098,7 +4086,7 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="117" t="s">
+      <c r="A2" s="118" t="s">
         <v>0</v>
       </c>
       <c r="B2">
@@ -4106,16 +4094,16 @@
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="117"/>
+      <c r="A3" s="118"/>
       <c r="B3">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="117"/>
+      <c r="A4" s="118"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="117"/>
+      <c r="A5" s="118"/>
       <c r="B5">
         <f>SUM(B2:B3)</f>
         <v>3</v>
@@ -4149,23 +4137,23 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="128" t="s">
+      <c r="A2" s="120" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="183" t="s">
+      <c r="B2" s="121" t="s">
         <v>65</v>
       </c>
-      <c r="C2" s="184"/>
-      <c r="D2" s="184"/>
-      <c r="E2" s="184"/>
-      <c r="F2" s="184"/>
-      <c r="G2" s="184"/>
-      <c r="H2" s="184"/>
-      <c r="I2" s="185"/>
-      <c r="J2" s="182"/>
+      <c r="C2" s="122"/>
+      <c r="D2" s="122"/>
+      <c r="E2" s="122"/>
+      <c r="F2" s="122"/>
+      <c r="G2" s="122"/>
+      <c r="H2" s="122"/>
+      <c r="I2" s="123"/>
+      <c r="J2" s="131"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="128"/>
+      <c r="A3" s="120"/>
       <c r="B3" s="3">
         <v>28</v>
       </c>
@@ -4190,7 +4178,7 @@
       <c r="I3" s="3">
         <v>35</v>
       </c>
-      <c r="J3" s="182"/>
+      <c r="J3" s="131"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
@@ -4198,22 +4186,22 @@
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="128" t="s">
+      <c r="A8" s="120" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="183" t="s">
+      <c r="B8" s="121" t="s">
         <v>65</v>
       </c>
-      <c r="C8" s="184"/>
-      <c r="D8" s="184"/>
-      <c r="E8" s="184"/>
-      <c r="F8" s="184"/>
-      <c r="G8" s="184"/>
-      <c r="H8" s="184"/>
-      <c r="I8" s="185"/>
+      <c r="C8" s="122"/>
+      <c r="D8" s="122"/>
+      <c r="E8" s="122"/>
+      <c r="F8" s="122"/>
+      <c r="G8" s="122"/>
+      <c r="H8" s="122"/>
+      <c r="I8" s="123"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="128"/>
+      <c r="A9" s="120"/>
       <c r="B9" s="3">
         <v>28</v>
       </c>
@@ -4240,7 +4228,7 @@
       </c>
     </row>
     <row r="10" spans="1:10" ht="15" x14ac:dyDescent="0.3">
-      <c r="A10" s="128"/>
+      <c r="A10" s="120"/>
       <c r="B10" s="4">
         <v>1</v>
       </c>
@@ -4267,7 +4255,7 @@
       </c>
     </row>
     <row r="11" spans="1:10" ht="15" x14ac:dyDescent="0.3">
-      <c r="A11" s="128"/>
+      <c r="A11" s="120"/>
       <c r="B11" s="4">
         <v>1</v>
       </c>
@@ -4294,7 +4282,7 @@
       </c>
     </row>
     <row r="12" spans="1:10" ht="15" x14ac:dyDescent="0.3">
-      <c r="A12" s="128"/>
+      <c r="A12" s="120"/>
       <c r="B12" s="4"/>
       <c r="C12" s="5"/>
       <c r="D12" s="4">
@@ -4307,7 +4295,7 @@
       <c r="I12" s="5"/>
     </row>
     <row r="13" spans="1:10" ht="15" x14ac:dyDescent="0.3">
-      <c r="A13" s="128"/>
+      <c r="A13" s="120"/>
       <c r="B13" s="4"/>
       <c r="C13" s="5"/>
       <c r="D13" s="4"/>
@@ -4320,7 +4308,7 @@
       <c r="I13" s="5"/>
     </row>
     <row r="14" spans="1:10" ht="15" x14ac:dyDescent="0.3">
-      <c r="A14" s="128"/>
+      <c r="A14" s="120"/>
       <c r="B14" s="4"/>
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
@@ -4333,7 +4321,7 @@
       <c r="I14" s="6"/>
     </row>
     <row r="15" spans="1:10" ht="15" x14ac:dyDescent="0.3">
-      <c r="A15" s="128"/>
+      <c r="A15" s="120"/>
       <c r="B15" s="4"/>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
@@ -4346,7 +4334,7 @@
       <c r="I15" s="6"/>
     </row>
     <row r="16" spans="1:10" ht="15" x14ac:dyDescent="0.3">
-      <c r="A16" s="128"/>
+      <c r="A16" s="120"/>
       <c r="B16" s="4"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
@@ -4362,16 +4350,16 @@
       <c r="A20" s="1"/>
     </row>
     <row r="22" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A22" s="128" t="s">
+      <c r="A22" s="120" t="s">
         <v>0</v>
       </c>
-      <c r="B22" s="194" t="s">
+      <c r="B22" s="129" t="s">
         <v>110</v>
       </c>
-      <c r="C22" s="176" t="s">
+      <c r="C22" s="140" t="s">
         <v>111</v>
       </c>
-      <c r="D22" s="157" t="s">
+      <c r="D22" s="146" t="s">
         <v>112</v>
       </c>
       <c r="E22" s="56"/>
@@ -4384,10 +4372,10 @@
       <c r="L22" s="58"/>
     </row>
     <row r="23" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A23" s="128"/>
-      <c r="B23" s="195"/>
-      <c r="C23" s="177"/>
-      <c r="D23" s="158"/>
+      <c r="A23" s="120"/>
+      <c r="B23" s="130"/>
+      <c r="C23" s="141"/>
+      <c r="D23" s="147"/>
       <c r="E23" s="3">
         <v>28</v>
       </c>
@@ -4414,7 +4402,7 @@
       </c>
     </row>
     <row r="24" spans="1:29" ht="15" x14ac:dyDescent="0.3">
-      <c r="A24" s="128"/>
+      <c r="A24" s="120"/>
       <c r="C24" s="36">
         <v>2040</v>
       </c>
@@ -4447,7 +4435,7 @@
       </c>
     </row>
     <row r="25" spans="1:29" ht="15" x14ac:dyDescent="0.3">
-      <c r="A25" s="128"/>
+      <c r="A25" s="120"/>
       <c r="B25" s="47"/>
       <c r="C25" s="48">
         <v>980</v>
@@ -4481,7 +4469,7 @@
       </c>
     </row>
     <row r="26" spans="1:29" ht="15" x14ac:dyDescent="0.3">
-      <c r="A26" s="128"/>
+      <c r="A26" s="120"/>
       <c r="B26" s="46"/>
       <c r="C26" s="36">
         <v>96</v>
@@ -4501,7 +4489,7 @@
       <c r="L26" s="5"/>
     </row>
     <row r="27" spans="1:29" ht="15" x14ac:dyDescent="0.3">
-      <c r="A27" s="128"/>
+      <c r="A27" s="120"/>
       <c r="B27" s="46">
         <v>16501</v>
       </c>
@@ -4523,7 +4511,7 @@
       <c r="L27" s="5"/>
     </row>
     <row r="28" spans="1:29" ht="15" x14ac:dyDescent="0.3">
-      <c r="A28" s="128"/>
+      <c r="A28" s="120"/>
       <c r="B28" s="46"/>
       <c r="C28" s="36">
         <v>96</v>
@@ -4543,7 +4531,7 @@
       <c r="L28" s="6"/>
     </row>
     <row r="29" spans="1:29" ht="15" x14ac:dyDescent="0.3">
-      <c r="A29" s="128"/>
+      <c r="A29" s="120"/>
       <c r="B29" s="46"/>
       <c r="C29" s="36">
         <v>96</v>
@@ -4563,7 +4551,7 @@
       <c r="L29" s="6"/>
     </row>
     <row r="30" spans="1:29" ht="15" x14ac:dyDescent="0.3">
-      <c r="A30" s="128"/>
+      <c r="A30" s="120"/>
       <c r="B30" s="46"/>
       <c r="C30" s="36">
         <v>96</v>
@@ -4583,7 +4571,7 @@
       <c r="L30" s="6"/>
     </row>
     <row r="31" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A31" s="128"/>
+      <c r="A31" s="120"/>
       <c r="C31">
         <f>SUM(C24:C30)</f>
         <v>3500</v>
@@ -4600,26 +4588,26 @@
       </c>
     </row>
     <row r="32" spans="1:29" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A32" s="128"/>
-      <c r="B32" s="191"/>
-      <c r="C32" s="192"/>
-      <c r="D32" s="192"/>
-      <c r="E32" s="192"/>
-      <c r="F32" s="192"/>
-      <c r="G32" s="192"/>
-      <c r="H32" s="192"/>
-      <c r="I32" s="192"/>
-      <c r="J32" s="192"/>
-      <c r="K32" s="192"/>
-      <c r="L32" s="192"/>
-      <c r="M32" s="192"/>
-      <c r="N32" s="192"/>
-      <c r="O32" s="192"/>
-      <c r="P32" s="192"/>
-      <c r="Q32" s="192"/>
-      <c r="R32" s="192"/>
-      <c r="S32" s="192"/>
-      <c r="T32" s="193"/>
+      <c r="A32" s="120"/>
+      <c r="B32" s="137"/>
+      <c r="C32" s="138"/>
+      <c r="D32" s="138"/>
+      <c r="E32" s="138"/>
+      <c r="F32" s="138"/>
+      <c r="G32" s="138"/>
+      <c r="H32" s="138"/>
+      <c r="I32" s="138"/>
+      <c r="J32" s="138"/>
+      <c r="K32" s="138"/>
+      <c r="L32" s="138"/>
+      <c r="M32" s="138"/>
+      <c r="N32" s="138"/>
+      <c r="O32" s="138"/>
+      <c r="P32" s="138"/>
+      <c r="Q32" s="138"/>
+      <c r="R32" s="138"/>
+      <c r="S32" s="138"/>
+      <c r="T32" s="139"/>
       <c r="U32" s="15"/>
       <c r="V32" s="15"/>
       <c r="W32" s="26"/>
@@ -4638,37 +4626,37 @@
       </c>
     </row>
     <row r="39" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A39" s="128" t="s">
+      <c r="A39" s="120" t="s">
         <v>0</v>
       </c>
-      <c r="B39" s="194" t="s">
+      <c r="B39" s="129" t="s">
         <v>110</v>
       </c>
-      <c r="C39" s="136" t="s">
+      <c r="C39" s="127" t="s">
         <v>80</v>
       </c>
-      <c r="D39" s="196" t="s">
+      <c r="D39" s="125" t="s">
         <v>81</v>
       </c>
-      <c r="E39" s="136" t="s">
+      <c r="E39" s="127" t="s">
         <v>82</v>
       </c>
-      <c r="F39" s="136" t="s">
+      <c r="F39" s="127" t="s">
         <v>83</v>
       </c>
-      <c r="G39" s="134" t="s">
+      <c r="G39" s="150" t="s">
         <v>84</v>
       </c>
-      <c r="H39" s="136" t="s">
+      <c r="H39" s="127" t="s">
         <v>85</v>
       </c>
-      <c r="I39" s="134" t="s">
+      <c r="I39" s="150" t="s">
         <v>86</v>
       </c>
-      <c r="J39" s="136" t="s">
+      <c r="J39" s="127" t="s">
         <v>87</v>
       </c>
-      <c r="K39" s="136" t="s">
+      <c r="K39" s="127" t="s">
         <v>88</v>
       </c>
       <c r="L39" s="56"/>
@@ -4679,49 +4667,49 @@
       <c r="Q39" s="57"/>
       <c r="R39" s="57"/>
       <c r="S39" s="58"/>
-      <c r="T39" s="136" t="s">
+      <c r="T39" s="127" t="s">
         <v>89</v>
       </c>
-      <c r="U39" s="136" t="s">
+      <c r="U39" s="127" t="s">
         <v>90</v>
       </c>
-      <c r="V39" s="176" t="s">
+      <c r="V39" s="140" t="s">
         <v>111</v>
       </c>
-      <c r="W39" s="174" t="s">
+      <c r="W39" s="165" t="s">
         <v>91</v>
       </c>
-      <c r="X39" s="178" t="s">
+      <c r="X39" s="142" t="s">
         <v>92</v>
       </c>
-      <c r="Y39" s="180" t="s">
+      <c r="Y39" s="144" t="s">
         <v>93</v>
       </c>
-      <c r="Z39" s="132" t="s">
+      <c r="Z39" s="167" t="s">
         <v>94</v>
       </c>
-      <c r="AA39" s="172" t="s">
+      <c r="AA39" s="148" t="s">
         <v>95</v>
       </c>
-      <c r="AB39" s="172" t="s">
+      <c r="AB39" s="148" t="s">
         <v>96</v>
       </c>
-      <c r="AC39" s="157" t="s">
+      <c r="AC39" s="146" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="40" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A40" s="128"/>
-      <c r="B40" s="195"/>
-      <c r="C40" s="137"/>
-      <c r="D40" s="197"/>
-      <c r="E40" s="137"/>
-      <c r="F40" s="137"/>
-      <c r="G40" s="135"/>
-      <c r="H40" s="137"/>
-      <c r="I40" s="135"/>
-      <c r="J40" s="137"/>
-      <c r="K40" s="137"/>
+      <c r="A40" s="120"/>
+      <c r="B40" s="130"/>
+      <c r="C40" s="128"/>
+      <c r="D40" s="126"/>
+      <c r="E40" s="128"/>
+      <c r="F40" s="128"/>
+      <c r="G40" s="151"/>
+      <c r="H40" s="128"/>
+      <c r="I40" s="151"/>
+      <c r="J40" s="128"/>
+      <c r="K40" s="128"/>
       <c r="L40" s="3">
         <v>28</v>
       </c>
@@ -4746,42 +4734,42 @@
       <c r="S40" s="3">
         <v>35</v>
       </c>
-      <c r="T40" s="137"/>
-      <c r="U40" s="137"/>
-      <c r="V40" s="177"/>
-      <c r="W40" s="175"/>
-      <c r="X40" s="179"/>
-      <c r="Y40" s="181"/>
-      <c r="Z40" s="133"/>
-      <c r="AA40" s="173"/>
-      <c r="AB40" s="173"/>
-      <c r="AC40" s="158"/>
+      <c r="T40" s="128"/>
+      <c r="U40" s="128"/>
+      <c r="V40" s="141"/>
+      <c r="W40" s="166"/>
+      <c r="X40" s="143"/>
+      <c r="Y40" s="145"/>
+      <c r="Z40" s="168"/>
+      <c r="AA40" s="149"/>
+      <c r="AB40" s="149"/>
+      <c r="AC40" s="147"/>
     </row>
     <row r="41" spans="1:29" ht="28" x14ac:dyDescent="0.3">
-      <c r="A41" s="128"/>
-      <c r="C41" s="159">
+      <c r="A41" s="120"/>
+      <c r="C41" s="152">
         <v>91338035</v>
       </c>
       <c r="D41" s="7">
         <v>532325</v>
       </c>
-      <c r="E41" s="159" t="s">
+      <c r="E41" s="152" t="s">
         <v>97</v>
       </c>
-      <c r="F41" s="162" t="s">
+      <c r="F41" s="155" t="s">
         <v>98</v>
       </c>
-      <c r="G41" s="159" t="s">
+      <c r="G41" s="152" t="s">
         <v>98</v>
       </c>
-      <c r="H41" s="159"/>
-      <c r="I41" s="162" t="s">
+      <c r="H41" s="152"/>
+      <c r="I41" s="155" t="s">
         <v>99</v>
       </c>
-      <c r="J41" s="162" t="s">
+      <c r="J41" s="155" t="s">
         <v>100</v>
       </c>
-      <c r="K41" s="162" t="s">
+      <c r="K41" s="155" t="s">
         <v>125</v>
       </c>
       <c r="L41" s="4">
@@ -4821,13 +4809,13 @@
       <c r="W41" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="X41" s="165" t="s">
+      <c r="X41" s="158" t="s">
         <v>102</v>
       </c>
       <c r="Y41" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="Z41" s="167">
+      <c r="Z41" s="160">
         <v>43171</v>
       </c>
       <c r="AA41" s="12"/>
@@ -4838,19 +4826,19 @@
       </c>
     </row>
     <row r="42" spans="1:29" s="45" customFormat="1" ht="28" x14ac:dyDescent="0.3">
-      <c r="A42" s="128"/>
+      <c r="A42" s="120"/>
       <c r="B42" s="47"/>
-      <c r="C42" s="160"/>
+      <c r="C42" s="153"/>
       <c r="D42" s="48">
         <v>532326</v>
       </c>
-      <c r="E42" s="160"/>
-      <c r="F42" s="163"/>
-      <c r="G42" s="160"/>
-      <c r="H42" s="160"/>
-      <c r="I42" s="163"/>
-      <c r="J42" s="163"/>
-      <c r="K42" s="163"/>
+      <c r="E42" s="153"/>
+      <c r="F42" s="156"/>
+      <c r="G42" s="153"/>
+      <c r="H42" s="153"/>
+      <c r="I42" s="156"/>
+      <c r="J42" s="156"/>
+      <c r="K42" s="156"/>
       <c r="L42" s="49">
         <v>1</v>
       </c>
@@ -4888,11 +4876,11 @@
       <c r="W42" s="52" t="s">
         <v>104</v>
       </c>
-      <c r="X42" s="166"/>
+      <c r="X42" s="159"/>
       <c r="Y42" s="53" t="s">
         <v>105</v>
       </c>
-      <c r="Z42" s="168"/>
+      <c r="Z42" s="161"/>
       <c r="AA42" s="54"/>
       <c r="AB42" s="54"/>
       <c r="AC42" s="55">
@@ -4901,19 +4889,19 @@
       </c>
     </row>
     <row r="43" spans="1:29" ht="15" x14ac:dyDescent="0.3">
-      <c r="A43" s="128"/>
+      <c r="A43" s="120"/>
       <c r="B43" s="46"/>
-      <c r="C43" s="160"/>
+      <c r="C43" s="153"/>
       <c r="D43" s="7">
         <v>533180</v>
       </c>
-      <c r="E43" s="160"/>
-      <c r="F43" s="163"/>
-      <c r="G43" s="160"/>
-      <c r="H43" s="160"/>
-      <c r="I43" s="163"/>
-      <c r="J43" s="163"/>
-      <c r="K43" s="163" t="s">
+      <c r="E43" s="153"/>
+      <c r="F43" s="156"/>
+      <c r="G43" s="153"/>
+      <c r="H43" s="153"/>
+      <c r="I43" s="156"/>
+      <c r="J43" s="156"/>
+      <c r="K43" s="156" t="s">
         <v>126</v>
       </c>
       <c r="L43" s="4"/>
@@ -4939,11 +4927,11 @@
       <c r="W43" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="X43" s="166"/>
-      <c r="Y43" s="170" t="s">
+      <c r="X43" s="159"/>
+      <c r="Y43" s="163" t="s">
         <v>107</v>
       </c>
-      <c r="Z43" s="168"/>
+      <c r="Z43" s="161"/>
       <c r="AA43" s="12"/>
       <c r="AB43" s="12"/>
       <c r="AC43" s="13">
@@ -4952,21 +4940,21 @@
       </c>
     </row>
     <row r="44" spans="1:29" ht="15" x14ac:dyDescent="0.3">
-      <c r="A44" s="128"/>
+      <c r="A44" s="120"/>
       <c r="B44" s="46">
         <v>16501</v>
       </c>
-      <c r="C44" s="160"/>
+      <c r="C44" s="153"/>
       <c r="D44" s="7">
         <v>533181</v>
       </c>
-      <c r="E44" s="160"/>
-      <c r="F44" s="163"/>
-      <c r="G44" s="160"/>
-      <c r="H44" s="160"/>
-      <c r="I44" s="163"/>
-      <c r="J44" s="163"/>
-      <c r="K44" s="163"/>
+      <c r="E44" s="153"/>
+      <c r="F44" s="156"/>
+      <c r="G44" s="153"/>
+      <c r="H44" s="153"/>
+      <c r="I44" s="156"/>
+      <c r="J44" s="156"/>
+      <c r="K44" s="156"/>
       <c r="L44" s="4"/>
       <c r="M44" s="5"/>
       <c r="N44" s="4"/>
@@ -4990,9 +4978,9 @@
       <c r="W44" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="X44" s="166"/>
-      <c r="Y44" s="171"/>
-      <c r="Z44" s="168"/>
+      <c r="X44" s="159"/>
+      <c r="Y44" s="164"/>
+      <c r="Z44" s="161"/>
       <c r="AA44" s="12"/>
       <c r="AB44" s="12"/>
       <c r="AC44" s="13">
@@ -5001,19 +4989,19 @@
       </c>
     </row>
     <row r="45" spans="1:29" ht="15" x14ac:dyDescent="0.3">
-      <c r="A45" s="128"/>
+      <c r="A45" s="120"/>
       <c r="B45" s="46"/>
-      <c r="C45" s="160"/>
+      <c r="C45" s="153"/>
       <c r="D45" s="7">
         <v>533182</v>
       </c>
-      <c r="E45" s="160"/>
-      <c r="F45" s="163"/>
-      <c r="G45" s="160"/>
-      <c r="H45" s="160"/>
-      <c r="I45" s="163"/>
-      <c r="J45" s="163"/>
-      <c r="K45" s="163"/>
+      <c r="E45" s="153"/>
+      <c r="F45" s="156"/>
+      <c r="G45" s="153"/>
+      <c r="H45" s="153"/>
+      <c r="I45" s="156"/>
+      <c r="J45" s="156"/>
+      <c r="K45" s="156"/>
       <c r="L45" s="4"/>
       <c r="M45" s="5"/>
       <c r="N45" s="5"/>
@@ -5037,9 +5025,9 @@
       <c r="W45" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="X45" s="166"/>
-      <c r="Y45" s="171"/>
-      <c r="Z45" s="168"/>
+      <c r="X45" s="159"/>
+      <c r="Y45" s="164"/>
+      <c r="Z45" s="161"/>
       <c r="AA45" s="12"/>
       <c r="AB45" s="12"/>
       <c r="AC45" s="13">
@@ -5048,19 +5036,19 @@
       </c>
     </row>
     <row r="46" spans="1:29" ht="15" x14ac:dyDescent="0.3">
-      <c r="A46" s="128"/>
+      <c r="A46" s="120"/>
       <c r="B46" s="46"/>
-      <c r="C46" s="160"/>
+      <c r="C46" s="153"/>
       <c r="D46" s="36">
         <v>533183</v>
       </c>
-      <c r="E46" s="160"/>
-      <c r="F46" s="163"/>
-      <c r="G46" s="160"/>
-      <c r="H46" s="160"/>
-      <c r="I46" s="163"/>
-      <c r="J46" s="163"/>
-      <c r="K46" s="163"/>
+      <c r="E46" s="153"/>
+      <c r="F46" s="156"/>
+      <c r="G46" s="153"/>
+      <c r="H46" s="153"/>
+      <c r="I46" s="156"/>
+      <c r="J46" s="156"/>
+      <c r="K46" s="156"/>
       <c r="L46" s="4"/>
       <c r="M46" s="5"/>
       <c r="N46" s="5"/>
@@ -5084,9 +5072,9 @@
       <c r="W46" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="X46" s="166"/>
-      <c r="Y46" s="171"/>
-      <c r="Z46" s="168"/>
+      <c r="X46" s="159"/>
+      <c r="Y46" s="164"/>
+      <c r="Z46" s="161"/>
       <c r="AA46" s="12"/>
       <c r="AB46" s="12"/>
       <c r="AC46" s="13">
@@ -5095,19 +5083,19 @@
       </c>
     </row>
     <row r="47" spans="1:29" ht="15" x14ac:dyDescent="0.3">
-      <c r="A47" s="128"/>
+      <c r="A47" s="120"/>
       <c r="B47" s="46"/>
-      <c r="C47" s="161"/>
+      <c r="C47" s="154"/>
       <c r="D47" s="36">
         <v>533184</v>
       </c>
-      <c r="E47" s="161"/>
-      <c r="F47" s="164"/>
-      <c r="G47" s="161"/>
-      <c r="H47" s="161"/>
-      <c r="I47" s="164"/>
-      <c r="J47" s="164"/>
-      <c r="K47" s="164"/>
+      <c r="E47" s="154"/>
+      <c r="F47" s="157"/>
+      <c r="G47" s="154"/>
+      <c r="H47" s="154"/>
+      <c r="I47" s="157"/>
+      <c r="J47" s="157"/>
+      <c r="K47" s="157"/>
       <c r="L47" s="4"/>
       <c r="M47" s="5"/>
       <c r="N47" s="5"/>
@@ -5131,9 +5119,9 @@
       <c r="W47" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="X47" s="166"/>
-      <c r="Y47" s="171"/>
-      <c r="Z47" s="169"/>
+      <c r="X47" s="159"/>
+      <c r="Y47" s="164"/>
+      <c r="Z47" s="162"/>
       <c r="AA47" s="12"/>
       <c r="AB47" s="12"/>
       <c r="AC47" s="13">
@@ -5142,7 +5130,7 @@
       </c>
     </row>
     <row r="48" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A48" s="128"/>
+      <c r="A48" s="120"/>
       <c r="W48" s="14"/>
       <c r="X48" s="16"/>
       <c r="Y48" s="17"/>
@@ -5161,26 +5149,26 @@
       </c>
     </row>
     <row r="49" spans="1:29" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A49" s="128"/>
-      <c r="B49" s="191"/>
-      <c r="C49" s="192"/>
-      <c r="D49" s="192"/>
-      <c r="E49" s="192"/>
-      <c r="F49" s="192"/>
-      <c r="G49" s="192"/>
-      <c r="H49" s="192"/>
-      <c r="I49" s="192"/>
-      <c r="J49" s="192"/>
-      <c r="K49" s="192"/>
-      <c r="L49" s="192"/>
-      <c r="M49" s="192"/>
-      <c r="N49" s="192"/>
-      <c r="O49" s="192"/>
-      <c r="P49" s="192"/>
-      <c r="Q49" s="192"/>
-      <c r="R49" s="192"/>
-      <c r="S49" s="192"/>
-      <c r="T49" s="193"/>
+      <c r="A49" s="120"/>
+      <c r="B49" s="137"/>
+      <c r="C49" s="138"/>
+      <c r="D49" s="138"/>
+      <c r="E49" s="138"/>
+      <c r="F49" s="138"/>
+      <c r="G49" s="138"/>
+      <c r="H49" s="138"/>
+      <c r="I49" s="138"/>
+      <c r="J49" s="138"/>
+      <c r="K49" s="138"/>
+      <c r="L49" s="138"/>
+      <c r="M49" s="138"/>
+      <c r="N49" s="138"/>
+      <c r="O49" s="138"/>
+      <c r="P49" s="138"/>
+      <c r="Q49" s="138"/>
+      <c r="R49" s="138"/>
+      <c r="S49" s="138"/>
+      <c r="T49" s="139"/>
       <c r="U49" s="15"/>
       <c r="V49" s="15">
         <f>SUM(V41:V47)</f>
@@ -5227,67 +5215,67 @@
       </c>
     </row>
     <row r="63" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A63" s="128" t="s">
+      <c r="A63" s="120" t="s">
         <v>0</v>
       </c>
-      <c r="B63" s="194" t="s">
+      <c r="B63" s="129" t="s">
         <v>158</v>
       </c>
-      <c r="C63" s="136" t="s">
+      <c r="C63" s="127" t="s">
         <v>80</v>
       </c>
-      <c r="D63" s="196" t="s">
+      <c r="D63" s="125" t="s">
         <v>81</v>
       </c>
-      <c r="E63" s="136" t="s">
+      <c r="E63" s="127" t="s">
         <v>82</v>
       </c>
-      <c r="F63" s="136" t="s">
+      <c r="F63" s="127" t="s">
         <v>83</v>
       </c>
-      <c r="G63" s="134" t="s">
+      <c r="G63" s="150" t="s">
         <v>84</v>
       </c>
-      <c r="H63" s="136" t="s">
+      <c r="H63" s="127" t="s">
         <v>85</v>
       </c>
-      <c r="I63" s="134" t="s">
+      <c r="I63" s="150" t="s">
         <v>86</v>
       </c>
-      <c r="J63" s="136" t="s">
+      <c r="J63" s="127" t="s">
         <v>87</v>
       </c>
-      <c r="K63" s="136" t="s">
+      <c r="K63" s="127" t="s">
         <v>88</v>
       </c>
-      <c r="L63" s="136" t="s">
+      <c r="L63" s="127" t="s">
         <v>89</v>
       </c>
-      <c r="M63" s="136" t="s">
+      <c r="M63" s="127" t="s">
         <v>90</v>
       </c>
-      <c r="N63" s="176" t="s">
+      <c r="N63" s="140" t="s">
         <v>111</v>
       </c>
-      <c r="O63" s="174" t="s">
+      <c r="O63" s="165" t="s">
         <v>91</v>
       </c>
-      <c r="P63" s="178" t="s">
+      <c r="P63" s="142" t="s">
         <v>92</v>
       </c>
-      <c r="Q63" s="180" t="s">
+      <c r="Q63" s="144" t="s">
         <v>93</v>
       </c>
-      <c r="R63" s="132" t="s">
+      <c r="R63" s="167" t="s">
         <v>94</v>
       </c>
-      <c r="S63" s="172" t="s">
+      <c r="S63" s="148" t="s">
         <v>95</v>
       </c>
-      <c r="T63" s="172" t="s">
+      <c r="T63" s="148" t="s">
         <v>96</v>
       </c>
-      <c r="U63" s="157" t="s">
+      <c r="U63" s="146" t="s">
         <v>112</v>
       </c>
       <c r="V63" s="56"/>
@@ -5300,27 +5288,27 @@
       <c r="AC63" s="58"/>
     </row>
     <row r="64" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A64" s="128"/>
-      <c r="B64" s="195"/>
-      <c r="C64" s="137"/>
-      <c r="D64" s="197"/>
-      <c r="E64" s="137"/>
-      <c r="F64" s="137"/>
-      <c r="G64" s="135"/>
-      <c r="H64" s="137"/>
-      <c r="I64" s="135"/>
-      <c r="J64" s="137"/>
-      <c r="K64" s="137"/>
-      <c r="L64" s="137"/>
-      <c r="M64" s="137"/>
-      <c r="N64" s="177"/>
-      <c r="O64" s="175"/>
-      <c r="P64" s="179"/>
-      <c r="Q64" s="181"/>
-      <c r="R64" s="133"/>
-      <c r="S64" s="173"/>
-      <c r="T64" s="173"/>
-      <c r="U64" s="158"/>
+      <c r="A64" s="120"/>
+      <c r="B64" s="130"/>
+      <c r="C64" s="128"/>
+      <c r="D64" s="126"/>
+      <c r="E64" s="128"/>
+      <c r="F64" s="128"/>
+      <c r="G64" s="151"/>
+      <c r="H64" s="128"/>
+      <c r="I64" s="151"/>
+      <c r="J64" s="128"/>
+      <c r="K64" s="128"/>
+      <c r="L64" s="128"/>
+      <c r="M64" s="128"/>
+      <c r="N64" s="141"/>
+      <c r="O64" s="166"/>
+      <c r="P64" s="143"/>
+      <c r="Q64" s="145"/>
+      <c r="R64" s="168"/>
+      <c r="S64" s="149"/>
+      <c r="T64" s="149"/>
+      <c r="U64" s="147"/>
       <c r="V64" s="3">
         <v>28</v>
       </c>
@@ -5347,30 +5335,30 @@
       </c>
     </row>
     <row r="65" spans="1:29" ht="28" x14ac:dyDescent="0.3">
-      <c r="A65" s="128"/>
-      <c r="C65" s="159">
+      <c r="A65" s="120"/>
+      <c r="C65" s="152">
         <v>91338035</v>
       </c>
       <c r="D65" s="36">
         <v>532325</v>
       </c>
-      <c r="E65" s="159" t="s">
+      <c r="E65" s="152" t="s">
         <v>97</v>
       </c>
-      <c r="F65" s="162" t="s">
+      <c r="F65" s="155" t="s">
         <v>98</v>
       </c>
-      <c r="G65" s="159" t="s">
+      <c r="G65" s="152" t="s">
         <v>98</v>
       </c>
-      <c r="H65" s="159"/>
-      <c r="I65" s="162" t="s">
+      <c r="H65" s="152"/>
+      <c r="I65" s="155" t="s">
         <v>99</v>
       </c>
-      <c r="J65" s="162" t="s">
+      <c r="J65" s="155" t="s">
         <v>100</v>
       </c>
-      <c r="K65" s="162" t="s">
+      <c r="K65" s="155" t="s">
         <v>125</v>
       </c>
       <c r="L65" s="8">
@@ -5386,13 +5374,13 @@
       <c r="O65" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="P65" s="165" t="s">
+      <c r="P65" s="158" t="s">
         <v>102</v>
       </c>
       <c r="Q65" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="R65" s="167">
+      <c r="R65" s="160">
         <v>43171</v>
       </c>
       <c r="S65" s="12"/>
@@ -5427,19 +5415,19 @@
       </c>
     </row>
     <row r="66" spans="1:29" ht="28" x14ac:dyDescent="0.3">
-      <c r="A66" s="128"/>
+      <c r="A66" s="120"/>
       <c r="B66" s="47"/>
-      <c r="C66" s="160"/>
+      <c r="C66" s="153"/>
       <c r="D66" s="48">
         <v>532326</v>
       </c>
-      <c r="E66" s="160"/>
-      <c r="F66" s="163"/>
-      <c r="G66" s="160"/>
-      <c r="H66" s="160"/>
-      <c r="I66" s="163"/>
-      <c r="J66" s="163"/>
-      <c r="K66" s="163"/>
+      <c r="E66" s="153"/>
+      <c r="F66" s="156"/>
+      <c r="G66" s="153"/>
+      <c r="H66" s="153"/>
+      <c r="I66" s="156"/>
+      <c r="J66" s="156"/>
+      <c r="K66" s="156"/>
       <c r="L66" s="50">
         <v>10</v>
       </c>
@@ -5453,11 +5441,11 @@
       <c r="O66" s="52" t="s">
         <v>104</v>
       </c>
-      <c r="P66" s="166"/>
+      <c r="P66" s="159"/>
       <c r="Q66" s="53" t="s">
         <v>105</v>
       </c>
-      <c r="R66" s="168"/>
+      <c r="R66" s="161"/>
       <c r="S66" s="54"/>
       <c r="T66" s="54"/>
       <c r="U66" s="55">
@@ -5490,19 +5478,19 @@
       </c>
     </row>
     <row r="67" spans="1:29" ht="15" x14ac:dyDescent="0.3">
-      <c r="A67" s="128"/>
+      <c r="A67" s="120"/>
       <c r="B67" s="46"/>
-      <c r="C67" s="160"/>
+      <c r="C67" s="153"/>
       <c r="D67" s="36">
         <v>533180</v>
       </c>
-      <c r="E67" s="160"/>
-      <c r="F67" s="163"/>
-      <c r="G67" s="160"/>
-      <c r="H67" s="160"/>
-      <c r="I67" s="163"/>
-      <c r="J67" s="163"/>
-      <c r="K67" s="163" t="s">
+      <c r="E67" s="153"/>
+      <c r="F67" s="156"/>
+      <c r="G67" s="153"/>
+      <c r="H67" s="153"/>
+      <c r="I67" s="156"/>
+      <c r="J67" s="156"/>
+      <c r="K67" s="156" t="s">
         <v>126</v>
       </c>
       <c r="L67" s="8">
@@ -5518,11 +5506,11 @@
       <c r="O67" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="P67" s="166"/>
-      <c r="Q67" s="170" t="s">
+      <c r="P67" s="159"/>
+      <c r="Q67" s="163" t="s">
         <v>107</v>
       </c>
-      <c r="R67" s="168"/>
+      <c r="R67" s="161"/>
       <c r="S67" s="12"/>
       <c r="T67" s="12"/>
       <c r="U67" s="13">
@@ -5541,21 +5529,21 @@
       <c r="AC67" s="5"/>
     </row>
     <row r="68" spans="1:29" ht="15" x14ac:dyDescent="0.3">
-      <c r="A68" s="128"/>
+      <c r="A68" s="120"/>
       <c r="B68" s="46">
         <v>16501</v>
       </c>
-      <c r="C68" s="160"/>
+      <c r="C68" s="153"/>
       <c r="D68" s="36">
         <v>533181</v>
       </c>
-      <c r="E68" s="160"/>
-      <c r="F68" s="163"/>
-      <c r="G68" s="160"/>
-      <c r="H68" s="160"/>
-      <c r="I68" s="163"/>
-      <c r="J68" s="163"/>
-      <c r="K68" s="163"/>
+      <c r="E68" s="153"/>
+      <c r="F68" s="156"/>
+      <c r="G68" s="153"/>
+      <c r="H68" s="153"/>
+      <c r="I68" s="156"/>
+      <c r="J68" s="156"/>
+      <c r="K68" s="156"/>
       <c r="L68" s="8">
         <v>16</v>
       </c>
@@ -5569,9 +5557,9 @@
       <c r="O68" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="P68" s="166"/>
-      <c r="Q68" s="171"/>
-      <c r="R68" s="168"/>
+      <c r="P68" s="159"/>
+      <c r="Q68" s="164"/>
+      <c r="R68" s="161"/>
       <c r="S68" s="12"/>
       <c r="T68" s="12"/>
       <c r="U68" s="13">
@@ -5590,19 +5578,19 @@
       <c r="AC68" s="5"/>
     </row>
     <row r="69" spans="1:29" ht="15" x14ac:dyDescent="0.3">
-      <c r="A69" s="128"/>
+      <c r="A69" s="120"/>
       <c r="B69" s="46"/>
-      <c r="C69" s="160"/>
+      <c r="C69" s="153"/>
       <c r="D69" s="36">
         <v>533182</v>
       </c>
-      <c r="E69" s="160"/>
-      <c r="F69" s="163"/>
-      <c r="G69" s="160"/>
-      <c r="H69" s="160"/>
-      <c r="I69" s="163"/>
-      <c r="J69" s="163"/>
-      <c r="K69" s="163"/>
+      <c r="E69" s="153"/>
+      <c r="F69" s="156"/>
+      <c r="G69" s="153"/>
+      <c r="H69" s="153"/>
+      <c r="I69" s="156"/>
+      <c r="J69" s="156"/>
+      <c r="K69" s="156"/>
       <c r="L69" s="8">
         <v>16</v>
       </c>
@@ -5616,9 +5604,9 @@
       <c r="O69" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="P69" s="166"/>
-      <c r="Q69" s="171"/>
-      <c r="R69" s="168"/>
+      <c r="P69" s="159"/>
+      <c r="Q69" s="164"/>
+      <c r="R69" s="161"/>
       <c r="S69" s="12"/>
       <c r="T69" s="12"/>
       <c r="U69" s="13">
@@ -5637,19 +5625,19 @@
       <c r="AC69" s="6"/>
     </row>
     <row r="70" spans="1:29" ht="15" x14ac:dyDescent="0.3">
-      <c r="A70" s="128"/>
+      <c r="A70" s="120"/>
       <c r="B70" s="46"/>
-      <c r="C70" s="160"/>
+      <c r="C70" s="153"/>
       <c r="D70" s="36">
         <v>533183</v>
       </c>
-      <c r="E70" s="160"/>
-      <c r="F70" s="163"/>
-      <c r="G70" s="160"/>
-      <c r="H70" s="160"/>
-      <c r="I70" s="163"/>
-      <c r="J70" s="163"/>
-      <c r="K70" s="163"/>
+      <c r="E70" s="153"/>
+      <c r="F70" s="156"/>
+      <c r="G70" s="153"/>
+      <c r="H70" s="153"/>
+      <c r="I70" s="156"/>
+      <c r="J70" s="156"/>
+      <c r="K70" s="156"/>
       <c r="L70" s="8">
         <v>16</v>
       </c>
@@ -5663,9 +5651,9 @@
       <c r="O70" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="P70" s="166"/>
-      <c r="Q70" s="171"/>
-      <c r="R70" s="168"/>
+      <c r="P70" s="159"/>
+      <c r="Q70" s="164"/>
+      <c r="R70" s="161"/>
       <c r="S70" s="12"/>
       <c r="T70" s="12"/>
       <c r="U70" s="13">
@@ -5684,19 +5672,19 @@
       <c r="AC70" s="6"/>
     </row>
     <row r="71" spans="1:29" ht="15" x14ac:dyDescent="0.3">
-      <c r="A71" s="128"/>
+      <c r="A71" s="120"/>
       <c r="B71" s="46"/>
-      <c r="C71" s="161"/>
+      <c r="C71" s="154"/>
       <c r="D71" s="36">
         <v>533184</v>
       </c>
-      <c r="E71" s="161"/>
-      <c r="F71" s="164"/>
-      <c r="G71" s="161"/>
-      <c r="H71" s="161"/>
-      <c r="I71" s="164"/>
-      <c r="J71" s="164"/>
-      <c r="K71" s="164"/>
+      <c r="E71" s="154"/>
+      <c r="F71" s="157"/>
+      <c r="G71" s="154"/>
+      <c r="H71" s="154"/>
+      <c r="I71" s="157"/>
+      <c r="J71" s="157"/>
+      <c r="K71" s="157"/>
       <c r="L71" s="8">
         <v>16</v>
       </c>
@@ -5710,9 +5698,9 @@
       <c r="O71" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="P71" s="166"/>
-      <c r="Q71" s="171"/>
-      <c r="R71" s="169"/>
+      <c r="P71" s="159"/>
+      <c r="Q71" s="164"/>
+      <c r="R71" s="162"/>
       <c r="S71" s="12"/>
       <c r="T71" s="12"/>
       <c r="U71" s="13">
@@ -5731,7 +5719,7 @@
       <c r="AC71" s="6"/>
     </row>
     <row r="72" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A72" s="128"/>
+      <c r="A72" s="120"/>
       <c r="S72" s="18">
         <f>SUM(S65:S71)</f>
         <v>0</v>
@@ -5746,7 +5734,7 @@
       </c>
     </row>
     <row r="73" spans="1:29" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A73" s="128"/>
+      <c r="A73" s="120"/>
       <c r="B73" s="46"/>
       <c r="C73" s="46"/>
       <c r="D73" s="46"/>
@@ -5789,16 +5777,16 @@
       </c>
     </row>
     <row r="78" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A78" s="128" t="s">
+      <c r="A78" s="120" t="s">
         <v>0</v>
       </c>
-      <c r="B78" s="190" t="s">
+      <c r="B78" s="136" t="s">
         <v>139</v>
       </c>
-      <c r="C78" s="190" t="s">
+      <c r="C78" s="136" t="s">
         <v>140</v>
       </c>
-      <c r="D78" s="190" t="s">
+      <c r="D78" s="136" t="s">
         <v>141</v>
       </c>
       <c r="E78" s="38" t="s">
@@ -5824,10 +5812,10 @@
       </c>
     </row>
     <row r="79" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A79" s="128"/>
-      <c r="B79" s="190"/>
-      <c r="C79" s="190"/>
-      <c r="D79" s="190"/>
+      <c r="A79" s="120"/>
+      <c r="B79" s="136"/>
+      <c r="C79" s="136"/>
+      <c r="D79" s="136"/>
       <c r="E79" s="4" t="s">
         <v>143</v>
       </c>
@@ -5851,10 +5839,10 @@
       </c>
     </row>
     <row r="80" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A80" s="128"/>
-      <c r="B80" s="187"/>
-      <c r="C80" s="187"/>
-      <c r="D80" s="187"/>
+      <c r="A80" s="120"/>
+      <c r="B80" s="133"/>
+      <c r="C80" s="133"/>
+      <c r="D80" s="133"/>
       <c r="E80" s="4" t="s">
         <v>144</v>
       </c>
@@ -5878,14 +5866,14 @@
       </c>
     </row>
     <row r="81" spans="1:14" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A81" s="128"/>
-      <c r="B81" s="186" t="s">
+      <c r="A81" s="120"/>
+      <c r="B81" s="132" t="s">
         <v>145</v>
       </c>
       <c r="C81" s="42" t="s">
         <v>146</v>
       </c>
-      <c r="D81" s="186">
+      <c r="D81" s="132">
         <v>2129</v>
       </c>
       <c r="E81" s="42" t="s">
@@ -5917,12 +5905,12 @@
       </c>
     </row>
     <row r="82" spans="1:14" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A82" s="128"/>
-      <c r="B82" s="187"/>
+      <c r="A82" s="120"/>
+      <c r="B82" s="133"/>
       <c r="C82" s="43" t="s">
         <v>148</v>
       </c>
-      <c r="D82" s="187"/>
+      <c r="D82" s="133"/>
       <c r="E82" s="42" t="s">
         <v>147</v>
       </c>
@@ -5952,7 +5940,7 @@
       </c>
     </row>
     <row r="83" spans="1:14" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A83" s="128"/>
+      <c r="A83" s="120"/>
       <c r="B83" s="44" t="s">
         <v>149</v>
       </c>
@@ -5991,14 +5979,14 @@
       </c>
     </row>
     <row r="84" spans="1:14" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A84" s="128"/>
-      <c r="B84" s="186" t="s">
+      <c r="A84" s="120"/>
+      <c r="B84" s="132" t="s">
         <v>151</v>
       </c>
       <c r="C84" s="43" t="s">
         <v>152</v>
       </c>
-      <c r="D84" s="188">
+      <c r="D84" s="134">
         <v>2129</v>
       </c>
       <c r="E84" s="42" t="s">
@@ -6030,12 +6018,12 @@
       </c>
     </row>
     <row r="85" spans="1:14" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A85" s="128"/>
-      <c r="B85" s="187"/>
+      <c r="A85" s="120"/>
+      <c r="B85" s="133"/>
       <c r="C85" s="43" t="s">
         <v>150</v>
       </c>
-      <c r="D85" s="189"/>
+      <c r="D85" s="135"/>
       <c r="E85" s="42" t="s">
         <v>147</v>
       </c>
@@ -6072,7 +6060,7 @@
       </c>
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A89" s="128" t="s">
+      <c r="A89" s="120" t="s">
         <v>0</v>
       </c>
       <c r="L89">
@@ -6088,7 +6076,7 @@
       </c>
     </row>
     <row r="90" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A90" s="128"/>
+      <c r="A90" s="120"/>
       <c r="L90">
         <v>2300</v>
       </c>
@@ -6098,7 +6086,7 @@
       </c>
     </row>
     <row r="91" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A91" s="128"/>
+      <c r="A91" s="120"/>
       <c r="L91">
         <v>1600</v>
       </c>
@@ -6131,7 +6119,7 @@
       </c>
     </row>
     <row r="94" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A94" s="128" t="s">
+      <c r="A94" s="120" t="s">
         <v>0</v>
       </c>
       <c r="B94" s="78"/>
@@ -6142,50 +6130,50 @@
       <c r="G94" s="78"/>
     </row>
     <row r="95" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A95" s="128"/>
+      <c r="A95" s="120"/>
     </row>
     <row r="96" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A96" s="128"/>
+      <c r="A96" s="120"/>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="B98" s="119">
+      <c r="B98" s="117">
         <v>35</v>
       </c>
-      <c r="C98" s="119">
+      <c r="C98" s="117">
         <v>36</v>
       </c>
-      <c r="D98" s="119">
+      <c r="D98" s="117">
         <v>37</v>
       </c>
-      <c r="E98" s="119">
+      <c r="E98" s="117">
         <v>38</v>
       </c>
-      <c r="F98" s="119">
+      <c r="F98" s="117">
         <v>39</v>
       </c>
-      <c r="G98" s="119">
+      <c r="G98" s="117">
         <v>40</v>
       </c>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A99" s="128" t="s">
+      <c r="A99" s="120" t="s">
         <v>0</v>
       </c>
-      <c r="B99" s="119"/>
-      <c r="C99" s="119"/>
-      <c r="D99" s="119"/>
-      <c r="E99" s="119"/>
-      <c r="F99" s="119"/>
-      <c r="G99" s="119"/>
+      <c r="B99" s="117"/>
+      <c r="C99" s="117"/>
+      <c r="D99" s="117"/>
+      <c r="E99" s="117"/>
+      <c r="F99" s="117"/>
+      <c r="G99" s="117"/>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A100" s="128"/>
+      <c r="A100" s="120"/>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A101" s="128"/>
+      <c r="A101" s="120"/>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
@@ -6196,7 +6184,7 @@
       </c>
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A104" s="128" t="s">
+      <c r="A104" s="120" t="s">
         <v>0</v>
       </c>
       <c r="B104" s="78">
@@ -6219,10 +6207,10 @@
       </c>
     </row>
     <row r="105" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A105" s="128"/>
+      <c r="A105" s="120"/>
     </row>
     <row r="106" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A106" s="128"/>
+      <c r="A106" s="120"/>
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
@@ -6251,7 +6239,7 @@
       </c>
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A110" s="128" t="s">
+      <c r="A110" s="120" t="s">
         <v>0</v>
       </c>
       <c r="B110" s="4" t="s">
@@ -6277,7 +6265,7 @@
       </c>
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A111" s="128"/>
+      <c r="A111" s="120"/>
       <c r="B111" s="4" t="s">
         <v>144</v>
       </c>
@@ -6301,7 +6289,7 @@
       </c>
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A112" s="128"/>
+      <c r="A112" s="120"/>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A127" s="1" t="s">
@@ -6318,7 +6306,7 @@
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A128" s="128" t="s">
+      <c r="A128" s="120" t="s">
         <v>0</v>
       </c>
       <c r="B128" t="s">
@@ -6332,7 +6320,7 @@
       </c>
     </row>
     <row r="129" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A129" s="128"/>
+      <c r="A129" s="120"/>
       <c r="B129" t="s">
         <v>188</v>
       </c>
@@ -6344,7 +6332,7 @@
       </c>
     </row>
     <row r="130" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A130" s="128"/>
+      <c r="A130" s="120"/>
       <c r="B130" t="s">
         <v>188</v>
       </c>
@@ -6376,7 +6364,7 @@
       </c>
     </row>
     <row r="134" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A134" s="128" t="s">
+      <c r="A134" s="120" t="s">
         <v>0</v>
       </c>
       <c r="B134" t="s">
@@ -6396,7 +6384,7 @@
       </c>
     </row>
     <row r="135" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A135" s="128"/>
+      <c r="A135" s="120"/>
       <c r="B135" t="s">
         <v>188</v>
       </c>
@@ -6414,7 +6402,7 @@
       </c>
     </row>
     <row r="136" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A136" s="128"/>
+      <c r="A136" s="120"/>
       <c r="B136" t="s">
         <v>188</v>
       </c>
@@ -6467,7 +6455,7 @@
       </c>
     </row>
     <row r="139" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A139" s="128" t="s">
+      <c r="A139" s="120" t="s">
         <v>0</v>
       </c>
       <c r="B139" t="s">
@@ -6502,7 +6490,7 @@
       </c>
     </row>
     <row r="140" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A140" s="128"/>
+      <c r="A140" s="120"/>
       <c r="B140" t="s">
         <v>188</v>
       </c>
@@ -6535,7 +6523,7 @@
       </c>
     </row>
     <row r="141" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A141" s="128"/>
+      <c r="A141" s="120"/>
       <c r="B141" t="s">
         <v>188</v>
       </c>
@@ -6573,54 +6561,54 @@
       </c>
     </row>
     <row r="145" spans="1:11" ht="13.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A145" s="128" t="s">
+      <c r="A145" s="120" t="s">
         <v>0</v>
       </c>
-      <c r="B145" s="131" t="s">
+      <c r="B145" s="197" t="s">
         <v>200</v>
       </c>
-      <c r="C145" s="130" t="s">
+      <c r="C145" s="196" t="s">
         <v>206</v>
       </c>
-      <c r="D145" s="130"/>
-      <c r="E145" s="130"/>
+      <c r="D145" s="196"/>
+      <c r="E145" s="196"/>
     </row>
     <row r="146" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A146" s="128"/>
-      <c r="B146" s="131"/>
-      <c r="C146" s="129" t="s">
+      <c r="A146" s="120"/>
+      <c r="B146" s="197"/>
+      <c r="C146" s="124" t="s">
         <v>176</v>
       </c>
-      <c r="D146" s="129" t="s">
+      <c r="D146" s="124" t="s">
         <v>177</v>
       </c>
-      <c r="E146" s="129"/>
+      <c r="E146" s="124"/>
     </row>
     <row r="147" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A147" s="128"/>
-      <c r="B147" s="131"/>
-      <c r="C147" s="129"/>
-      <c r="D147" s="129"/>
-      <c r="E147" s="129"/>
+      <c r="A147" s="120"/>
+      <c r="B147" s="197"/>
+      <c r="C147" s="124"/>
+      <c r="D147" s="124"/>
+      <c r="E147" s="124"/>
     </row>
     <row r="148" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A148" s="77"/>
-      <c r="B148" s="131"/>
-      <c r="C148" s="129" t="s">
+      <c r="B148" s="197"/>
+      <c r="C148" s="124" t="s">
         <v>197</v>
       </c>
-      <c r="D148" s="129" t="s">
+      <c r="D148" s="124" t="s">
         <v>198</v>
       </c>
-      <c r="E148" s="129" t="s">
+      <c r="E148" s="124" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="149" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A149" s="77"/>
-      <c r="C149" s="129"/>
-      <c r="D149" s="129"/>
-      <c r="E149" s="129"/>
+      <c r="C149" s="124"/>
+      <c r="D149" s="124"/>
+      <c r="E149" s="124"/>
     </row>
     <row r="150" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A150" s="79"/>
@@ -6640,30 +6628,30 @@
       </c>
     </row>
     <row r="154" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A154" s="128" t="s">
+      <c r="A154" s="120" t="s">
         <v>0</v>
       </c>
-      <c r="B154" s="129" t="s">
+      <c r="B154" s="124" t="s">
         <v>207</v>
       </c>
-      <c r="C154" s="129" t="s">
+      <c r="C154" s="124" t="s">
         <v>187</v>
       </c>
-      <c r="D154" s="119" t="s">
+      <c r="D154" s="117" t="s">
         <v>65</v>
       </c>
-      <c r="E154" s="119"/>
-      <c r="F154" s="119"/>
-      <c r="G154" s="119"/>
-      <c r="H154" s="119"/>
-      <c r="I154" s="119"/>
-      <c r="J154" s="129"/>
-      <c r="K154" s="129"/>
+      <c r="E154" s="117"/>
+      <c r="F154" s="117"/>
+      <c r="G154" s="117"/>
+      <c r="H154" s="117"/>
+      <c r="I154" s="117"/>
+      <c r="J154" s="124"/>
+      <c r="K154" s="124"/>
     </row>
     <row r="155" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A155" s="128"/>
-      <c r="B155" s="129"/>
-      <c r="C155" s="129"/>
+      <c r="A155" s="120"/>
+      <c r="B155" s="124"/>
+      <c r="C155" s="124"/>
       <c r="D155">
         <v>35</v>
       </c>
@@ -6682,11 +6670,11 @@
       <c r="I155">
         <v>40</v>
       </c>
-      <c r="J155" s="129"/>
-      <c r="K155" s="129"/>
+      <c r="J155" s="124"/>
+      <c r="K155" s="124"/>
     </row>
     <row r="156" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A156" s="128"/>
+      <c r="A156" s="120"/>
     </row>
     <row r="159" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A159" s="1" t="s">
@@ -6694,34 +6682,34 @@
       </c>
     </row>
     <row r="160" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A160" s="128" t="s">
+      <c r="A160" s="120" t="s">
         <v>0</v>
       </c>
-      <c r="B160" s="129" t="s">
+      <c r="B160" s="124" t="s">
         <v>222</v>
       </c>
-      <c r="C160" s="129" t="s">
+      <c r="C160" s="124" t="s">
         <v>187</v>
       </c>
-      <c r="D160" s="119" t="s">
+      <c r="D160" s="117" t="s">
         <v>65</v>
       </c>
-      <c r="E160" s="119"/>
-      <c r="F160" s="119"/>
-      <c r="G160" s="119"/>
-      <c r="H160" s="119"/>
-      <c r="I160" s="119"/>
-      <c r="J160" s="129" t="s">
+      <c r="E160" s="117"/>
+      <c r="F160" s="117"/>
+      <c r="G160" s="117"/>
+      <c r="H160" s="117"/>
+      <c r="I160" s="117"/>
+      <c r="J160" s="124" t="s">
         <v>168</v>
       </c>
-      <c r="K160" s="129" t="s">
+      <c r="K160" s="124" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="161" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A161" s="128"/>
-      <c r="B161" s="129"/>
-      <c r="C161" s="129"/>
+      <c r="A161" s="120"/>
+      <c r="B161" s="124"/>
+      <c r="C161" s="124"/>
       <c r="D161">
         <v>35</v>
       </c>
@@ -6740,17 +6728,17 @@
       <c r="I161">
         <v>40</v>
       </c>
-      <c r="J161" s="129"/>
-      <c r="K161" s="129"/>
+      <c r="J161" s="124"/>
+      <c r="K161" s="124"/>
     </row>
     <row r="162" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A162" s="128"/>
+      <c r="A162" s="120"/>
     </row>
     <row r="167" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B167" s="129" t="s">
+      <c r="B167" s="124" t="s">
         <v>196</v>
       </c>
-      <c r="C167" s="129" t="s">
+      <c r="C167" s="124" t="s">
         <v>187</v>
       </c>
       <c r="E167" s="78"/>
@@ -6760,10 +6748,10 @@
       </c>
       <c r="H167" s="78"/>
       <c r="I167" s="78"/>
-      <c r="J167" s="129" t="s">
+      <c r="J167" s="124" t="s">
         <v>192</v>
       </c>
-      <c r="K167" s="129" t="s">
+      <c r="K167" s="124" t="s">
         <v>193</v>
       </c>
     </row>
@@ -6771,8 +6759,8 @@
       <c r="A168" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="B168" s="129"/>
-      <c r="C168" s="129"/>
+      <c r="B168" s="124"/>
+      <c r="C168" s="124"/>
       <c r="D168">
         <v>35</v>
       </c>
@@ -6791,11 +6779,11 @@
       <c r="I168">
         <v>40</v>
       </c>
-      <c r="J168" s="129"/>
-      <c r="K168" s="129"/>
+      <c r="J168" s="124"/>
+      <c r="K168" s="124"/>
     </row>
     <row r="169" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A169" s="128" t="s">
+      <c r="A169" s="120" t="s">
         <v>0</v>
       </c>
       <c r="B169" t="s">
@@ -6830,7 +6818,7 @@
       </c>
     </row>
     <row r="170" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A170" s="128"/>
+      <c r="A170" s="120"/>
       <c r="B170" t="s">
         <v>188</v>
       </c>
@@ -6863,7 +6851,7 @@
       </c>
     </row>
     <row r="171" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A171" s="128"/>
+      <c r="A171" s="120"/>
       <c r="B171" t="s">
         <v>188</v>
       </c>
@@ -6900,90 +6888,90 @@
       <c r="A173" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="B173" s="142" t="s">
+      <c r="B173" s="173" t="s">
         <v>164</v>
       </c>
-      <c r="C173" s="144" t="s">
+      <c r="C173" s="175" t="s">
         <v>165</v>
       </c>
-      <c r="D173" s="146" t="s">
+      <c r="D173" s="177" t="s">
         <v>166</v>
       </c>
-      <c r="E173" s="148" t="s">
+      <c r="E173" s="179" t="s">
         <v>167</v>
       </c>
-      <c r="F173" s="148" t="s">
+      <c r="F173" s="179" t="s">
         <v>168</v>
       </c>
-      <c r="G173" s="150"/>
-      <c r="H173" s="148" t="s">
+      <c r="G173" s="181"/>
+      <c r="H173" s="179" t="s">
         <v>169</v>
       </c>
-      <c r="I173" s="151">
+      <c r="I173" s="182">
         <v>19</v>
       </c>
-      <c r="J173" s="151">
+      <c r="J173" s="182">
         <v>20</v>
       </c>
-      <c r="K173" s="151">
+      <c r="K173" s="182">
         <v>21</v>
       </c>
-      <c r="L173" s="151">
+      <c r="L173" s="182">
         <v>22</v>
       </c>
-      <c r="M173" s="151">
+      <c r="M173" s="182">
         <v>23</v>
       </c>
-      <c r="N173" s="151"/>
-      <c r="O173" s="148" t="s">
+      <c r="N173" s="182"/>
+      <c r="O173" s="179" t="s">
         <v>170</v>
       </c>
-      <c r="P173" s="148" t="s">
+      <c r="P173" s="179" t="s">
         <v>171</v>
       </c>
-      <c r="Q173" s="148" t="s">
+      <c r="Q173" s="179" t="s">
         <v>172</v>
       </c>
-      <c r="R173" s="148" t="s">
+      <c r="R173" s="179" t="s">
         <v>173</v>
       </c>
-      <c r="S173" s="148" t="s">
+      <c r="S173" s="179" t="s">
         <v>174</v>
       </c>
-      <c r="T173" s="153" t="s">
+      <c r="T173" s="184" t="s">
         <v>175</v>
       </c>
-      <c r="U173" s="154"/>
+      <c r="U173" s="185"/>
     </row>
     <row r="174" spans="1:21" ht="15" x14ac:dyDescent="0.3">
-      <c r="A174" s="128" t="s">
+      <c r="A174" s="120" t="s">
         <v>0</v>
       </c>
-      <c r="B174" s="143"/>
-      <c r="C174" s="145"/>
-      <c r="D174" s="147"/>
-      <c r="E174" s="149"/>
+      <c r="B174" s="174"/>
+      <c r="C174" s="176"/>
+      <c r="D174" s="178"/>
+      <c r="E174" s="180"/>
       <c r="F174" s="60"/>
       <c r="G174" s="60" t="s">
         <v>177</v>
       </c>
-      <c r="H174" s="149"/>
-      <c r="I174" s="149"/>
-      <c r="J174" s="149"/>
-      <c r="K174" s="149"/>
-      <c r="L174" s="149"/>
-      <c r="M174" s="149"/>
-      <c r="N174" s="149"/>
-      <c r="O174" s="152"/>
-      <c r="P174" s="149"/>
-      <c r="Q174" s="149"/>
-      <c r="R174" s="149"/>
-      <c r="S174" s="149"/>
-      <c r="T174" s="155"/>
-      <c r="U174" s="156"/>
+      <c r="H174" s="180"/>
+      <c r="I174" s="180"/>
+      <c r="J174" s="180"/>
+      <c r="K174" s="180"/>
+      <c r="L174" s="180"/>
+      <c r="M174" s="180"/>
+      <c r="N174" s="180"/>
+      <c r="O174" s="183"/>
+      <c r="P174" s="180"/>
+      <c r="Q174" s="180"/>
+      <c r="R174" s="180"/>
+      <c r="S174" s="180"/>
+      <c r="T174" s="186"/>
+      <c r="U174" s="187"/>
     </row>
     <row r="175" spans="1:21" ht="28" x14ac:dyDescent="0.3">
-      <c r="A175" s="128"/>
+      <c r="A175" s="120"/>
       <c r="B175" s="61" t="s">
         <v>178</v>
       </c>
@@ -7032,11 +7020,11 @@
         <f t="shared" ref="S175:S178" si="4">R175*Q175</f>
         <v>0</v>
       </c>
-      <c r="T175" s="138"/>
-      <c r="U175" s="139"/>
+      <c r="T175" s="169"/>
+      <c r="U175" s="170"/>
     </row>
     <row r="176" spans="1:21" ht="42" x14ac:dyDescent="0.3">
-      <c r="A176" s="128"/>
+      <c r="A176" s="120"/>
       <c r="B176" s="61" t="s">
         <v>178</v>
       </c>
@@ -7225,8 +7213,8 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="T179" s="140"/>
-      <c r="U179" s="141"/>
+      <c r="T179" s="171"/>
+      <c r="U179" s="172"/>
     </row>
     <row r="180" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A180" s="59"/>
@@ -7455,14 +7443,14 @@
       <c r="D223" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="E223" s="120" t="s">
+      <c r="E223" s="188" t="s">
         <v>237</v>
       </c>
-      <c r="F223" s="120"/>
-      <c r="G223" s="120"/>
-      <c r="H223" s="120"/>
-      <c r="I223" s="120"/>
-      <c r="J223" s="120"/>
+      <c r="F223" s="188"/>
+      <c r="G223" s="188"/>
+      <c r="H223" s="188"/>
+      <c r="I223" s="188"/>
+      <c r="J223" s="188"/>
     </row>
     <row r="224" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B224" s="101"/>
@@ -7490,10 +7478,10 @@
       </c>
     </row>
     <row r="225" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B225" s="121">
+      <c r="B225" s="189">
         <v>68637</v>
       </c>
-      <c r="C225" s="123" t="s">
+      <c r="C225" s="191" t="s">
         <v>239</v>
       </c>
       <c r="D225" s="104">
@@ -7519,14 +7507,14 @@
       </c>
     </row>
     <row r="226" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B226" s="122"/>
-      <c r="C226" s="124"/>
+      <c r="B226" s="190"/>
+      <c r="C226" s="192"/>
     </row>
     <row r="227" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B227" s="120">
+      <c r="B227" s="188">
         <v>68634</v>
       </c>
-      <c r="C227" s="125" t="s">
+      <c r="C227" s="193" t="s">
         <v>240</v>
       </c>
       <c r="D227" s="105" t="s">
@@ -7552,8 +7540,8 @@
       </c>
     </row>
     <row r="228" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B228" s="120"/>
-      <c r="C228" s="126"/>
+      <c r="B228" s="188"/>
+      <c r="C228" s="194"/>
       <c r="D228" s="106">
         <v>5896652</v>
       </c>
@@ -7577,8 +7565,8 @@
       </c>
     </row>
     <row r="229" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B229" s="120"/>
-      <c r="C229" s="127"/>
+      <c r="B229" s="188"/>
+      <c r="C229" s="195"/>
       <c r="D229" s="106">
         <v>5891652</v>
       </c>
@@ -7626,6 +7614,132 @@
     </row>
   </sheetData>
   <mergeCells count="150">
+    <mergeCell ref="E223:J223"/>
+    <mergeCell ref="B225:B226"/>
+    <mergeCell ref="C225:C226"/>
+    <mergeCell ref="B227:B229"/>
+    <mergeCell ref="C227:C229"/>
+    <mergeCell ref="G98:G99"/>
+    <mergeCell ref="A154:A156"/>
+    <mergeCell ref="D146:E147"/>
+    <mergeCell ref="C145:E145"/>
+    <mergeCell ref="A145:A147"/>
+    <mergeCell ref="B145:B148"/>
+    <mergeCell ref="C148:C149"/>
+    <mergeCell ref="D148:D149"/>
+    <mergeCell ref="E148:E149"/>
+    <mergeCell ref="A169:A171"/>
+    <mergeCell ref="B167:B168"/>
+    <mergeCell ref="C167:C168"/>
+    <mergeCell ref="J167:J168"/>
+    <mergeCell ref="K167:K168"/>
+    <mergeCell ref="B154:B155"/>
+    <mergeCell ref="C154:C155"/>
+    <mergeCell ref="J154:J155"/>
+    <mergeCell ref="K154:K155"/>
+    <mergeCell ref="D154:I154"/>
+    <mergeCell ref="A160:A162"/>
+    <mergeCell ref="B160:B161"/>
+    <mergeCell ref="C160:C161"/>
+    <mergeCell ref="D160:I160"/>
+    <mergeCell ref="J160:J161"/>
+    <mergeCell ref="K160:K161"/>
+    <mergeCell ref="R63:R64"/>
+    <mergeCell ref="G39:G40"/>
+    <mergeCell ref="C39:C40"/>
+    <mergeCell ref="T175:U175"/>
+    <mergeCell ref="T179:U179"/>
+    <mergeCell ref="A174:A176"/>
+    <mergeCell ref="B173:B174"/>
+    <mergeCell ref="C173:C174"/>
+    <mergeCell ref="D173:D174"/>
+    <mergeCell ref="E173:E174"/>
+    <mergeCell ref="F173:G173"/>
+    <mergeCell ref="H173:H174"/>
+    <mergeCell ref="I173:I174"/>
+    <mergeCell ref="J173:J174"/>
+    <mergeCell ref="K173:K174"/>
+    <mergeCell ref="L173:L174"/>
+    <mergeCell ref="M173:M174"/>
+    <mergeCell ref="N173:N174"/>
+    <mergeCell ref="O173:O174"/>
+    <mergeCell ref="P173:P174"/>
+    <mergeCell ref="Q173:Q174"/>
+    <mergeCell ref="R173:R174"/>
+    <mergeCell ref="S173:S174"/>
+    <mergeCell ref="T173:U174"/>
+    <mergeCell ref="U63:U64"/>
+    <mergeCell ref="C65:C71"/>
+    <mergeCell ref="E65:E71"/>
+    <mergeCell ref="F65:F71"/>
+    <mergeCell ref="G65:G71"/>
+    <mergeCell ref="H65:H71"/>
+    <mergeCell ref="I65:I71"/>
+    <mergeCell ref="J65:J71"/>
+    <mergeCell ref="K65:K66"/>
+    <mergeCell ref="P65:P71"/>
+    <mergeCell ref="R65:R71"/>
+    <mergeCell ref="K67:K71"/>
+    <mergeCell ref="Q67:Q71"/>
+    <mergeCell ref="S63:S64"/>
+    <mergeCell ref="O63:O64"/>
+    <mergeCell ref="N63:N64"/>
+    <mergeCell ref="M63:M64"/>
+    <mergeCell ref="L63:L64"/>
+    <mergeCell ref="K63:K64"/>
+    <mergeCell ref="J63:J64"/>
+    <mergeCell ref="I63:I64"/>
+    <mergeCell ref="H63:H64"/>
+    <mergeCell ref="G63:G64"/>
+    <mergeCell ref="F63:F64"/>
+    <mergeCell ref="AB39:AB40"/>
+    <mergeCell ref="AC39:AC40"/>
+    <mergeCell ref="C41:C47"/>
+    <mergeCell ref="E41:E47"/>
+    <mergeCell ref="F41:F47"/>
+    <mergeCell ref="G41:G47"/>
+    <mergeCell ref="H41:H47"/>
+    <mergeCell ref="I41:I47"/>
+    <mergeCell ref="J41:J47"/>
+    <mergeCell ref="X41:X47"/>
+    <mergeCell ref="Z41:Z47"/>
+    <mergeCell ref="K41:K42"/>
+    <mergeCell ref="K43:K47"/>
+    <mergeCell ref="AA39:AA40"/>
+    <mergeCell ref="Y43:Y47"/>
+    <mergeCell ref="V39:V40"/>
+    <mergeCell ref="W39:W40"/>
+    <mergeCell ref="X39:X40"/>
+    <mergeCell ref="Y39:Y40"/>
+    <mergeCell ref="Z39:Z40"/>
+    <mergeCell ref="J39:J40"/>
+    <mergeCell ref="K39:K40"/>
+    <mergeCell ref="T39:T40"/>
+    <mergeCell ref="U39:U40"/>
+    <mergeCell ref="J2:J3"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="A134:A136"/>
+    <mergeCell ref="A22:A32"/>
+    <mergeCell ref="B84:B85"/>
+    <mergeCell ref="D84:D85"/>
+    <mergeCell ref="A78:A85"/>
+    <mergeCell ref="B78:B80"/>
+    <mergeCell ref="C78:C80"/>
+    <mergeCell ref="D78:D80"/>
+    <mergeCell ref="B81:B82"/>
+    <mergeCell ref="D81:D82"/>
+    <mergeCell ref="B49:T49"/>
+    <mergeCell ref="A39:A49"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="P63:P64"/>
+    <mergeCell ref="Q63:Q64"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="T63:T64"/>
+    <mergeCell ref="B32:T32"/>
+    <mergeCell ref="H39:H40"/>
+    <mergeCell ref="I39:I40"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B8:I8"/>
     <mergeCell ref="A8:A16"/>
@@ -7650,132 +7764,6 @@
     <mergeCell ref="D98:D99"/>
     <mergeCell ref="E98:E99"/>
     <mergeCell ref="F98:F99"/>
-    <mergeCell ref="J2:J3"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="A134:A136"/>
-    <mergeCell ref="A22:A32"/>
-    <mergeCell ref="B84:B85"/>
-    <mergeCell ref="D84:D85"/>
-    <mergeCell ref="A78:A85"/>
-    <mergeCell ref="B78:B80"/>
-    <mergeCell ref="C78:C80"/>
-    <mergeCell ref="D78:D80"/>
-    <mergeCell ref="B81:B82"/>
-    <mergeCell ref="D81:D82"/>
-    <mergeCell ref="B49:T49"/>
-    <mergeCell ref="A39:A49"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="P63:P64"/>
-    <mergeCell ref="Q63:Q64"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="T63:T64"/>
-    <mergeCell ref="B32:T32"/>
-    <mergeCell ref="H39:H40"/>
-    <mergeCell ref="I39:I40"/>
-    <mergeCell ref="AB39:AB40"/>
-    <mergeCell ref="AC39:AC40"/>
-    <mergeCell ref="C41:C47"/>
-    <mergeCell ref="E41:E47"/>
-    <mergeCell ref="F41:F47"/>
-    <mergeCell ref="G41:G47"/>
-    <mergeCell ref="H41:H47"/>
-    <mergeCell ref="I41:I47"/>
-    <mergeCell ref="J41:J47"/>
-    <mergeCell ref="X41:X47"/>
-    <mergeCell ref="Z41:Z47"/>
-    <mergeCell ref="K41:K42"/>
-    <mergeCell ref="K43:K47"/>
-    <mergeCell ref="AA39:AA40"/>
-    <mergeCell ref="Y43:Y47"/>
-    <mergeCell ref="V39:V40"/>
-    <mergeCell ref="W39:W40"/>
-    <mergeCell ref="X39:X40"/>
-    <mergeCell ref="Y39:Y40"/>
-    <mergeCell ref="Z39:Z40"/>
-    <mergeCell ref="J39:J40"/>
-    <mergeCell ref="K39:K40"/>
-    <mergeCell ref="T39:T40"/>
-    <mergeCell ref="U39:U40"/>
-    <mergeCell ref="U63:U64"/>
-    <mergeCell ref="C65:C71"/>
-    <mergeCell ref="E65:E71"/>
-    <mergeCell ref="F65:F71"/>
-    <mergeCell ref="G65:G71"/>
-    <mergeCell ref="H65:H71"/>
-    <mergeCell ref="I65:I71"/>
-    <mergeCell ref="J65:J71"/>
-    <mergeCell ref="K65:K66"/>
-    <mergeCell ref="P65:P71"/>
-    <mergeCell ref="R65:R71"/>
-    <mergeCell ref="K67:K71"/>
-    <mergeCell ref="Q67:Q71"/>
-    <mergeCell ref="S63:S64"/>
-    <mergeCell ref="O63:O64"/>
-    <mergeCell ref="N63:N64"/>
-    <mergeCell ref="M63:M64"/>
-    <mergeCell ref="L63:L64"/>
-    <mergeCell ref="K63:K64"/>
-    <mergeCell ref="J63:J64"/>
-    <mergeCell ref="I63:I64"/>
-    <mergeCell ref="H63:H64"/>
-    <mergeCell ref="G63:G64"/>
-    <mergeCell ref="F63:F64"/>
-    <mergeCell ref="R63:R64"/>
-    <mergeCell ref="G39:G40"/>
-    <mergeCell ref="C39:C40"/>
-    <mergeCell ref="T175:U175"/>
-    <mergeCell ref="T179:U179"/>
-    <mergeCell ref="A174:A176"/>
-    <mergeCell ref="B173:B174"/>
-    <mergeCell ref="C173:C174"/>
-    <mergeCell ref="D173:D174"/>
-    <mergeCell ref="E173:E174"/>
-    <mergeCell ref="F173:G173"/>
-    <mergeCell ref="H173:H174"/>
-    <mergeCell ref="I173:I174"/>
-    <mergeCell ref="J173:J174"/>
-    <mergeCell ref="K173:K174"/>
-    <mergeCell ref="L173:L174"/>
-    <mergeCell ref="M173:M174"/>
-    <mergeCell ref="N173:N174"/>
-    <mergeCell ref="O173:O174"/>
-    <mergeCell ref="P173:P174"/>
-    <mergeCell ref="Q173:Q174"/>
-    <mergeCell ref="R173:R174"/>
-    <mergeCell ref="S173:S174"/>
-    <mergeCell ref="T173:U174"/>
-    <mergeCell ref="K167:K168"/>
-    <mergeCell ref="B154:B155"/>
-    <mergeCell ref="C154:C155"/>
-    <mergeCell ref="J154:J155"/>
-    <mergeCell ref="K154:K155"/>
-    <mergeCell ref="D154:I154"/>
-    <mergeCell ref="A160:A162"/>
-    <mergeCell ref="B160:B161"/>
-    <mergeCell ref="C160:C161"/>
-    <mergeCell ref="D160:I160"/>
-    <mergeCell ref="J160:J161"/>
-    <mergeCell ref="K160:K161"/>
-    <mergeCell ref="E223:J223"/>
-    <mergeCell ref="B225:B226"/>
-    <mergeCell ref="C225:C226"/>
-    <mergeCell ref="B227:B229"/>
-    <mergeCell ref="C227:C229"/>
-    <mergeCell ref="G98:G99"/>
-    <mergeCell ref="A154:A156"/>
-    <mergeCell ref="D146:E147"/>
-    <mergeCell ref="C145:E145"/>
-    <mergeCell ref="A145:A147"/>
-    <mergeCell ref="B145:B148"/>
-    <mergeCell ref="C148:C149"/>
-    <mergeCell ref="D148:D149"/>
-    <mergeCell ref="E148:E149"/>
-    <mergeCell ref="A169:A171"/>
-    <mergeCell ref="B167:B168"/>
-    <mergeCell ref="C167:C168"/>
-    <mergeCell ref="J167:J168"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7803,7 +7791,7 @@
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A2" s="128" t="s">
+      <c r="A2" s="120" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="91" t="s">
@@ -7818,47 +7806,47 @@
       </c>
       <c r="F2" s="90"/>
       <c r="G2" s="94"/>
-      <c r="H2" s="203" t="s">
+      <c r="H2" s="199" t="s">
         <v>224</v>
       </c>
-      <c r="I2" s="203"/>
-      <c r="J2" s="203"/>
-      <c r="K2" s="203"/>
-      <c r="L2" s="202" t="s">
+      <c r="I2" s="199"/>
+      <c r="J2" s="199"/>
+      <c r="K2" s="199"/>
+      <c r="L2" s="198" t="s">
         <v>229</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A3" s="128"/>
+      <c r="A3" s="120"/>
       <c r="B3" s="90"/>
       <c r="C3" s="99"/>
       <c r="D3" s="92" t="s">
         <v>226</v>
       </c>
       <c r="G3" s="95"/>
-      <c r="H3" s="202" t="s">
+      <c r="H3" s="198" t="s">
         <v>176</v>
       </c>
-      <c r="I3" s="206" t="s">
+      <c r="I3" s="202" t="s">
         <v>177</v>
       </c>
-      <c r="J3" s="206"/>
-      <c r="K3" s="206"/>
-      <c r="L3" s="202"/>
+      <c r="J3" s="202"/>
+      <c r="K3" s="202"/>
+      <c r="L3" s="198"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A4" s="128"/>
+      <c r="A4" s="120"/>
       <c r="B4" s="90"/>
       <c r="C4" s="99"/>
       <c r="D4" s="90"/>
       <c r="E4" s="90"/>
       <c r="F4" s="90"/>
       <c r="G4" s="94"/>
-      <c r="H4" s="202"/>
-      <c r="I4" s="206"/>
-      <c r="J4" s="206"/>
-      <c r="K4" s="206"/>
-      <c r="L4" s="202"/>
+      <c r="H4" s="198"/>
+      <c r="I4" s="202"/>
+      <c r="J4" s="202"/>
+      <c r="K4" s="202"/>
+      <c r="L4" s="198"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="77"/>
@@ -7868,30 +7856,30 @@
       <c r="E5" s="90"/>
       <c r="F5" s="90"/>
       <c r="G5" s="94"/>
-      <c r="H5" s="202" t="s">
+      <c r="H5" s="198" t="s">
         <v>197</v>
       </c>
-      <c r="I5" s="202" t="s">
+      <c r="I5" s="198" t="s">
         <v>198</v>
       </c>
-      <c r="J5" s="204" t="s">
+      <c r="J5" s="200" t="s">
         <v>199</v>
       </c>
-      <c r="K5" s="204"/>
-      <c r="L5" s="202"/>
+      <c r="K5" s="200"/>
+      <c r="L5" s="198"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="77"/>
-      <c r="E6" s="205" t="s">
+      <c r="E6" s="201" t="s">
         <v>228</v>
       </c>
-      <c r="F6" s="205"/>
+      <c r="F6" s="201"/>
       <c r="G6" s="94"/>
-      <c r="H6" s="202"/>
-      <c r="I6" s="202"/>
-      <c r="J6" s="204"/>
-      <c r="K6" s="204"/>
-      <c r="L6" s="202"/>
+      <c r="H6" s="198"/>
+      <c r="I6" s="198"/>
+      <c r="J6" s="200"/>
+      <c r="K6" s="200"/>
+      <c r="L6" s="198"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
@@ -7899,48 +7887,48 @@
       </c>
     </row>
     <row r="9" spans="1:12" ht="15.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="128" t="s">
+      <c r="A9" s="120" t="s">
         <v>0</v>
       </c>
-      <c r="B9" s="198" t="s">
+      <c r="B9" s="203" t="s">
         <v>243</v>
       </c>
-      <c r="C9" s="199"/>
-      <c r="D9" s="136" t="s">
+      <c r="C9" s="204"/>
+      <c r="D9" s="127" t="s">
         <v>83</v>
       </c>
-      <c r="E9" s="196" t="s">
+      <c r="E9" s="125" t="s">
         <v>81</v>
       </c>
-      <c r="F9" s="136" t="s">
+      <c r="F9" s="127" t="s">
         <v>88</v>
       </c>
-      <c r="G9" s="180" t="s">
+      <c r="G9" s="144" t="s">
         <v>93</v>
       </c>
-      <c r="H9" s="172" t="s">
+      <c r="H9" s="148" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A10" s="128"/>
-      <c r="B10" s="200"/>
-      <c r="C10" s="201"/>
-      <c r="D10" s="137"/>
-      <c r="E10" s="197"/>
-      <c r="F10" s="137"/>
-      <c r="G10" s="181"/>
-      <c r="H10" s="173"/>
+      <c r="A10" s="120"/>
+      <c r="B10" s="205"/>
+      <c r="C10" s="206"/>
+      <c r="D10" s="128"/>
+      <c r="E10" s="126"/>
+      <c r="F10" s="128"/>
+      <c r="G10" s="145"/>
+      <c r="H10" s="149"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A11" s="128"/>
-      <c r="D11" s="162" t="s">
+      <c r="A11" s="120"/>
+      <c r="D11" s="155" t="s">
         <v>98</v>
       </c>
       <c r="E11" s="36">
         <v>532325</v>
       </c>
-      <c r="F11" s="162" t="s">
+      <c r="F11" s="155" t="s">
         <v>125</v>
       </c>
       <c r="G11" s="11" t="s">
@@ -7949,82 +7937,82 @@
       <c r="H11" s="12"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A12" s="128"/>
+      <c r="A12" s="120"/>
       <c r="B12" s="47"/>
       <c r="C12" s="109"/>
-      <c r="D12" s="163"/>
+      <c r="D12" s="156"/>
       <c r="E12" s="48">
         <v>532326</v>
       </c>
-      <c r="F12" s="163"/>
+      <c r="F12" s="156"/>
       <c r="G12" s="53" t="s">
         <v>105</v>
       </c>
       <c r="H12" s="54"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A13" s="128"/>
+      <c r="A13" s="120"/>
       <c r="B13" s="95"/>
       <c r="C13" s="110"/>
-      <c r="D13" s="163"/>
+      <c r="D13" s="156"/>
       <c r="E13" s="36">
         <v>533180</v>
       </c>
-      <c r="F13" s="163" t="s">
+      <c r="F13" s="156" t="s">
         <v>126</v>
       </c>
-      <c r="G13" s="170" t="s">
+      <c r="G13" s="163" t="s">
         <v>107</v>
       </c>
       <c r="H13" s="12"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A14" s="128"/>
+      <c r="A14" s="120"/>
       <c r="C14" s="110"/>
-      <c r="D14" s="163"/>
+      <c r="D14" s="156"/>
       <c r="E14" s="36">
         <v>533181</v>
       </c>
-      <c r="F14" s="163"/>
-      <c r="G14" s="171"/>
+      <c r="F14" s="156"/>
+      <c r="G14" s="164"/>
       <c r="H14" s="12"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A15" s="128"/>
+      <c r="A15" s="120"/>
       <c r="B15" s="46"/>
       <c r="C15" s="110"/>
-      <c r="D15" s="163"/>
+      <c r="D15" s="156"/>
       <c r="E15" s="36">
         <v>533182</v>
       </c>
-      <c r="F15" s="163"/>
-      <c r="G15" s="171"/>
+      <c r="F15" s="156"/>
+      <c r="G15" s="164"/>
       <c r="H15" s="12"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A16" s="128"/>
+      <c r="A16" s="120"/>
       <c r="B16" s="46"/>
       <c r="C16" s="110"/>
-      <c r="D16" s="163"/>
+      <c r="D16" s="156"/>
       <c r="E16" s="36">
         <v>533183</v>
       </c>
-      <c r="F16" s="163"/>
-      <c r="G16" s="171"/>
+      <c r="F16" s="156"/>
+      <c r="G16" s="164"/>
       <c r="H16" s="12"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="128"/>
+      <c r="A17" s="120"/>
       <c r="B17" s="46">
         <v>16501</v>
       </c>
       <c r="C17" s="111"/>
-      <c r="D17" s="164"/>
+      <c r="D17" s="157"/>
       <c r="E17" s="36">
         <v>533184</v>
       </c>
-      <c r="F17" s="164"/>
-      <c r="G17" s="171"/>
+      <c r="F17" s="157"/>
+      <c r="G17" s="164"/>
       <c r="H17" s="12"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
@@ -8250,15 +8238,6 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="L2:L6"/>
-    <mergeCell ref="H2:K2"/>
-    <mergeCell ref="J5:K6"/>
-    <mergeCell ref="A2:A4"/>
-    <mergeCell ref="H3:H4"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="I3:K4"/>
     <mergeCell ref="F13:F17"/>
     <mergeCell ref="G9:G10"/>
     <mergeCell ref="H9:H10"/>
@@ -8270,6 +8249,15 @@
     <mergeCell ref="F9:F10"/>
     <mergeCell ref="D11:D17"/>
     <mergeCell ref="F11:F12"/>
+    <mergeCell ref="L2:L6"/>
+    <mergeCell ref="H2:K2"/>
+    <mergeCell ref="J5:K6"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="H3:H4"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="I3:K4"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8300,67 +8288,67 @@
       </c>
     </row>
     <row r="2" spans="1:29" ht="15.65" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="128" t="s">
+      <c r="A2" s="120" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="208" t="s">
+      <c r="B2" s="213" t="s">
         <v>242</v>
       </c>
-      <c r="C2" s="146" t="s">
+      <c r="C2" s="177" t="s">
         <v>165</v>
       </c>
-      <c r="D2" s="209" t="s">
+      <c r="D2" s="207" t="s">
         <v>166</v>
       </c>
-      <c r="E2" s="209" t="s">
+      <c r="E2" s="207" t="s">
         <v>167</v>
       </c>
-      <c r="F2" s="207" t="s">
+      <c r="F2" s="212" t="s">
         <v>168</v>
       </c>
-      <c r="G2" s="144"/>
-      <c r="H2" s="209" t="s">
+      <c r="G2" s="175"/>
+      <c r="H2" s="207" t="s">
         <v>169</v>
       </c>
-      <c r="I2" s="211" t="s">
+      <c r="I2" s="209" t="s">
         <v>230</v>
       </c>
-      <c r="J2" s="212"/>
-      <c r="K2" s="212"/>
-      <c r="L2" s="212"/>
-      <c r="M2" s="213"/>
+      <c r="J2" s="210"/>
+      <c r="K2" s="210"/>
+      <c r="L2" s="210"/>
+      <c r="M2" s="211"/>
       <c r="N2" s="100"/>
-      <c r="O2" s="209" t="s">
+      <c r="O2" s="207" t="s">
         <v>170</v>
       </c>
-      <c r="P2" s="209" t="s">
+      <c r="P2" s="207" t="s">
         <v>171</v>
       </c>
-      <c r="Q2" s="209" t="s">
+      <c r="Q2" s="207" t="s">
         <v>172</v>
       </c>
-      <c r="R2" s="209" t="s">
+      <c r="R2" s="207" t="s">
         <v>173</v>
       </c>
-      <c r="S2" s="209" t="s">
+      <c r="S2" s="207" t="s">
         <v>174</v>
       </c>
-      <c r="T2" s="153" t="s">
+      <c r="T2" s="184" t="s">
         <v>175</v>
       </c>
-      <c r="U2" s="154"/>
+      <c r="U2" s="185"/>
     </row>
     <row r="3" spans="1:29" ht="15" x14ac:dyDescent="0.3">
-      <c r="A3" s="128"/>
-      <c r="B3" s="208"/>
-      <c r="C3" s="147"/>
-      <c r="D3" s="210"/>
-      <c r="E3" s="210"/>
+      <c r="A3" s="120"/>
+      <c r="B3" s="213"/>
+      <c r="C3" s="178"/>
+      <c r="D3" s="208"/>
+      <c r="E3" s="208"/>
       <c r="F3" s="98"/>
       <c r="G3" s="98" t="s">
         <v>177</v>
       </c>
-      <c r="H3" s="210"/>
+      <c r="H3" s="208"/>
       <c r="I3" s="97">
         <v>19</v>
       </c>
@@ -8377,16 +8365,16 @@
         <v>23</v>
       </c>
       <c r="N3" s="97"/>
-      <c r="O3" s="210"/>
-      <c r="P3" s="210"/>
-      <c r="Q3" s="210"/>
-      <c r="R3" s="210"/>
-      <c r="S3" s="210"/>
-      <c r="T3" s="155"/>
-      <c r="U3" s="156"/>
+      <c r="O3" s="208"/>
+      <c r="P3" s="208"/>
+      <c r="Q3" s="208"/>
+      <c r="R3" s="208"/>
+      <c r="S3" s="208"/>
+      <c r="T3" s="186"/>
+      <c r="U3" s="187"/>
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A4" s="128"/>
+      <c r="A4" s="120"/>
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A5" s="77"/>
@@ -8400,37 +8388,37 @@
       </c>
     </row>
     <row r="14" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A14" s="128" t="s">
+      <c r="A14" s="120" t="s">
         <v>0</v>
       </c>
       <c r="B14" s="107" t="s">
         <v>241</v>
       </c>
-      <c r="C14" s="136" t="s">
+      <c r="C14" s="127" t="s">
         <v>80</v>
       </c>
-      <c r="D14" s="196" t="s">
+      <c r="D14" s="125" t="s">
         <v>81</v>
       </c>
-      <c r="E14" s="136" t="s">
+      <c r="E14" s="127" t="s">
         <v>82</v>
       </c>
-      <c r="F14" s="136" t="s">
+      <c r="F14" s="127" t="s">
         <v>83</v>
       </c>
-      <c r="G14" s="134" t="s">
+      <c r="G14" s="150" t="s">
         <v>84</v>
       </c>
-      <c r="H14" s="136" t="s">
+      <c r="H14" s="127" t="s">
         <v>85</v>
       </c>
-      <c r="I14" s="134" t="s">
+      <c r="I14" s="150" t="s">
         <v>86</v>
       </c>
-      <c r="J14" s="136" t="s">
+      <c r="J14" s="127" t="s">
         <v>87</v>
       </c>
-      <c r="K14" s="136" t="s">
+      <c r="K14" s="127" t="s">
         <v>88</v>
       </c>
       <c r="L14" s="56"/>
@@ -8441,49 +8429,49 @@
       <c r="Q14" s="57"/>
       <c r="R14" s="57"/>
       <c r="S14" s="58"/>
-      <c r="T14" s="136" t="s">
+      <c r="T14" s="127" t="s">
         <v>89</v>
       </c>
-      <c r="U14" s="136" t="s">
+      <c r="U14" s="127" t="s">
         <v>90</v>
       </c>
-      <c r="V14" s="176" t="s">
+      <c r="V14" s="140" t="s">
         <v>111</v>
       </c>
-      <c r="W14" s="174" t="s">
+      <c r="W14" s="165" t="s">
         <v>91</v>
       </c>
-      <c r="X14" s="178" t="s">
+      <c r="X14" s="142" t="s">
         <v>92</v>
       </c>
-      <c r="Y14" s="180" t="s">
+      <c r="Y14" s="144" t="s">
         <v>93</v>
       </c>
-      <c r="Z14" s="132" t="s">
+      <c r="Z14" s="167" t="s">
         <v>94</v>
       </c>
-      <c r="AA14" s="172" t="s">
+      <c r="AA14" s="148" t="s">
         <v>95</v>
       </c>
-      <c r="AB14" s="172" t="s">
+      <c r="AB14" s="148" t="s">
         <v>96</v>
       </c>
-      <c r="AC14" s="157" t="s">
+      <c r="AC14" s="146" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="15" spans="1:29" x14ac:dyDescent="0.3">
-      <c r="A15" s="128"/>
+      <c r="A15" s="120"/>
       <c r="B15" s="108"/>
-      <c r="C15" s="137"/>
-      <c r="D15" s="197"/>
-      <c r="E15" s="137"/>
-      <c r="F15" s="137"/>
-      <c r="G15" s="135"/>
-      <c r="H15" s="137"/>
-      <c r="I15" s="135"/>
-      <c r="J15" s="137"/>
-      <c r="K15" s="137"/>
+      <c r="C15" s="128"/>
+      <c r="D15" s="126"/>
+      <c r="E15" s="128"/>
+      <c r="F15" s="128"/>
+      <c r="G15" s="151"/>
+      <c r="H15" s="128"/>
+      <c r="I15" s="151"/>
+      <c r="J15" s="128"/>
+      <c r="K15" s="128"/>
       <c r="L15" s="3">
         <v>28</v>
       </c>
@@ -8508,42 +8496,42 @@
       <c r="S15" s="3">
         <v>35</v>
       </c>
-      <c r="T15" s="137"/>
-      <c r="U15" s="137"/>
-      <c r="V15" s="177"/>
-      <c r="W15" s="175"/>
-      <c r="X15" s="179"/>
-      <c r="Y15" s="181"/>
-      <c r="Z15" s="133"/>
-      <c r="AA15" s="173"/>
-      <c r="AB15" s="173"/>
-      <c r="AC15" s="158"/>
+      <c r="T15" s="128"/>
+      <c r="U15" s="128"/>
+      <c r="V15" s="141"/>
+      <c r="W15" s="166"/>
+      <c r="X15" s="143"/>
+      <c r="Y15" s="145"/>
+      <c r="Z15" s="168"/>
+      <c r="AA15" s="149"/>
+      <c r="AB15" s="149"/>
+      <c r="AC15" s="147"/>
     </row>
     <row r="16" spans="1:29" ht="28" x14ac:dyDescent="0.3">
-      <c r="A16" s="128"/>
-      <c r="C16" s="159">
+      <c r="A16" s="120"/>
+      <c r="C16" s="152">
         <v>91338035</v>
       </c>
       <c r="D16" s="36">
         <v>532325</v>
       </c>
-      <c r="E16" s="159" t="s">
+      <c r="E16" s="152" t="s">
         <v>97</v>
       </c>
-      <c r="F16" s="162" t="s">
+      <c r="F16" s="155" t="s">
         <v>98</v>
       </c>
-      <c r="G16" s="159" t="s">
+      <c r="G16" s="152" t="s">
         <v>98</v>
       </c>
-      <c r="H16" s="159"/>
-      <c r="I16" s="162" t="s">
+      <c r="H16" s="152"/>
+      <c r="I16" s="155" t="s">
         <v>99</v>
       </c>
-      <c r="J16" s="162" t="s">
+      <c r="J16" s="155" t="s">
         <v>100</v>
       </c>
-      <c r="K16" s="162" t="s">
+      <c r="K16" s="155" t="s">
         <v>125</v>
       </c>
       <c r="L16" s="102">
@@ -8583,13 +8571,13 @@
       <c r="W16" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="X16" s="165" t="s">
+      <c r="X16" s="158" t="s">
         <v>102</v>
       </c>
       <c r="Y16" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="Z16" s="167">
+      <c r="Z16" s="160">
         <v>43171</v>
       </c>
       <c r="AA16" s="12"/>
@@ -8600,19 +8588,19 @@
       </c>
     </row>
     <row r="17" spans="1:32" ht="28" x14ac:dyDescent="0.3">
-      <c r="A17" s="128"/>
+      <c r="A17" s="120"/>
       <c r="B17" s="47"/>
-      <c r="C17" s="160"/>
+      <c r="C17" s="153"/>
       <c r="D17" s="48">
         <v>532326</v>
       </c>
-      <c r="E17" s="160"/>
-      <c r="F17" s="163"/>
-      <c r="G17" s="160"/>
-      <c r="H17" s="160"/>
-      <c r="I17" s="163"/>
-      <c r="J17" s="163"/>
-      <c r="K17" s="163"/>
+      <c r="E17" s="153"/>
+      <c r="F17" s="156"/>
+      <c r="G17" s="153"/>
+      <c r="H17" s="153"/>
+      <c r="I17" s="156"/>
+      <c r="J17" s="156"/>
+      <c r="K17" s="156"/>
       <c r="L17" s="49">
         <v>1</v>
       </c>
@@ -8650,11 +8638,11 @@
       <c r="W17" s="52" t="s">
         <v>104</v>
       </c>
-      <c r="X17" s="166"/>
+      <c r="X17" s="159"/>
       <c r="Y17" s="53" t="s">
         <v>105</v>
       </c>
-      <c r="Z17" s="168"/>
+      <c r="Z17" s="161"/>
       <c r="AA17" s="54"/>
       <c r="AB17" s="54"/>
       <c r="AC17" s="55">
@@ -8663,19 +8651,19 @@
       </c>
     </row>
     <row r="18" spans="1:32" ht="15" x14ac:dyDescent="0.3">
-      <c r="A18" s="128"/>
+      <c r="A18" s="120"/>
       <c r="B18" s="46"/>
-      <c r="C18" s="160"/>
+      <c r="C18" s="153"/>
       <c r="D18" s="36">
         <v>533180</v>
       </c>
-      <c r="E18" s="160"/>
-      <c r="F18" s="163"/>
-      <c r="G18" s="160"/>
-      <c r="H18" s="160"/>
-      <c r="I18" s="163"/>
-      <c r="J18" s="163"/>
-      <c r="K18" s="163" t="s">
+      <c r="E18" s="153"/>
+      <c r="F18" s="156"/>
+      <c r="G18" s="153"/>
+      <c r="H18" s="153"/>
+      <c r="I18" s="156"/>
+      <c r="J18" s="156"/>
+      <c r="K18" s="156" t="s">
         <v>126</v>
       </c>
       <c r="L18" s="102"/>
@@ -8701,11 +8689,11 @@
       <c r="W18" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="X18" s="166"/>
-      <c r="Y18" s="170" t="s">
+      <c r="X18" s="159"/>
+      <c r="Y18" s="163" t="s">
         <v>107</v>
       </c>
-      <c r="Z18" s="168"/>
+      <c r="Z18" s="161"/>
       <c r="AA18" s="12"/>
       <c r="AB18" s="12"/>
       <c r="AC18" s="13">
@@ -8714,21 +8702,21 @@
       </c>
     </row>
     <row r="19" spans="1:32" ht="15" x14ac:dyDescent="0.3">
-      <c r="A19" s="128"/>
+      <c r="A19" s="120"/>
       <c r="B19" s="46">
         <v>16501</v>
       </c>
-      <c r="C19" s="160"/>
+      <c r="C19" s="153"/>
       <c r="D19" s="36">
         <v>533181</v>
       </c>
-      <c r="E19" s="160"/>
-      <c r="F19" s="163"/>
-      <c r="G19" s="160"/>
-      <c r="H19" s="160"/>
-      <c r="I19" s="163"/>
-      <c r="J19" s="163"/>
-      <c r="K19" s="163"/>
+      <c r="E19" s="153"/>
+      <c r="F19" s="156"/>
+      <c r="G19" s="153"/>
+      <c r="H19" s="153"/>
+      <c r="I19" s="156"/>
+      <c r="J19" s="156"/>
+      <c r="K19" s="156"/>
       <c r="L19" s="102"/>
       <c r="M19" s="5"/>
       <c r="N19" s="102"/>
@@ -8752,9 +8740,9 @@
       <c r="W19" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="X19" s="166"/>
-      <c r="Y19" s="171"/>
-      <c r="Z19" s="168"/>
+      <c r="X19" s="159"/>
+      <c r="Y19" s="164"/>
+      <c r="Z19" s="161"/>
       <c r="AA19" s="12"/>
       <c r="AB19" s="12"/>
       <c r="AC19" s="13">
@@ -8763,19 +8751,19 @@
       </c>
     </row>
     <row r="20" spans="1:32" ht="15" x14ac:dyDescent="0.3">
-      <c r="A20" s="128"/>
+      <c r="A20" s="120"/>
       <c r="B20" s="46"/>
-      <c r="C20" s="160"/>
+      <c r="C20" s="153"/>
       <c r="D20" s="36">
         <v>533182</v>
       </c>
-      <c r="E20" s="160"/>
-      <c r="F20" s="163"/>
-      <c r="G20" s="160"/>
-      <c r="H20" s="160"/>
-      <c r="I20" s="163"/>
-      <c r="J20" s="163"/>
-      <c r="K20" s="163"/>
+      <c r="E20" s="153"/>
+      <c r="F20" s="156"/>
+      <c r="G20" s="153"/>
+      <c r="H20" s="153"/>
+      <c r="I20" s="156"/>
+      <c r="J20" s="156"/>
+      <c r="K20" s="156"/>
       <c r="L20" s="102"/>
       <c r="M20" s="5"/>
       <c r="N20" s="5"/>
@@ -8799,9 +8787,9 @@
       <c r="W20" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="X20" s="166"/>
-      <c r="Y20" s="171"/>
-      <c r="Z20" s="168"/>
+      <c r="X20" s="159"/>
+      <c r="Y20" s="164"/>
+      <c r="Z20" s="161"/>
       <c r="AA20" s="12"/>
       <c r="AB20" s="12"/>
       <c r="AC20" s="13">
@@ -8810,19 +8798,19 @@
       </c>
     </row>
     <row r="21" spans="1:32" ht="15" x14ac:dyDescent="0.3">
-      <c r="A21" s="128"/>
+      <c r="A21" s="120"/>
       <c r="B21" s="46"/>
-      <c r="C21" s="160"/>
+      <c r="C21" s="153"/>
       <c r="D21" s="36">
         <v>533183</v>
       </c>
-      <c r="E21" s="160"/>
-      <c r="F21" s="163"/>
-      <c r="G21" s="160"/>
-      <c r="H21" s="160"/>
-      <c r="I21" s="163"/>
-      <c r="J21" s="163"/>
-      <c r="K21" s="163"/>
+      <c r="E21" s="153"/>
+      <c r="F21" s="156"/>
+      <c r="G21" s="153"/>
+      <c r="H21" s="153"/>
+      <c r="I21" s="156"/>
+      <c r="J21" s="156"/>
+      <c r="K21" s="156"/>
       <c r="L21" s="102"/>
       <c r="M21" s="5"/>
       <c r="N21" s="5"/>
@@ -8846,9 +8834,9 @@
       <c r="W21" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="X21" s="166"/>
-      <c r="Y21" s="171"/>
-      <c r="Z21" s="168"/>
+      <c r="X21" s="159"/>
+      <c r="Y21" s="164"/>
+      <c r="Z21" s="161"/>
       <c r="AA21" s="12"/>
       <c r="AB21" s="12"/>
       <c r="AC21" s="13">
@@ -8857,19 +8845,19 @@
       </c>
     </row>
     <row r="22" spans="1:32" ht="15" x14ac:dyDescent="0.3">
-      <c r="A22" s="128"/>
+      <c r="A22" s="120"/>
       <c r="B22" s="46"/>
-      <c r="C22" s="161"/>
+      <c r="C22" s="154"/>
       <c r="D22" s="36">
         <v>533184</v>
       </c>
-      <c r="E22" s="161"/>
-      <c r="F22" s="164"/>
-      <c r="G22" s="161"/>
-      <c r="H22" s="161"/>
-      <c r="I22" s="164"/>
-      <c r="J22" s="164"/>
-      <c r="K22" s="164"/>
+      <c r="E22" s="154"/>
+      <c r="F22" s="157"/>
+      <c r="G22" s="154"/>
+      <c r="H22" s="154"/>
+      <c r="I22" s="157"/>
+      <c r="J22" s="157"/>
+      <c r="K22" s="157"/>
       <c r="L22" s="102"/>
       <c r="M22" s="5"/>
       <c r="N22" s="5"/>
@@ -8893,9 +8881,9 @@
       <c r="W22" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="X22" s="166"/>
-      <c r="Y22" s="171"/>
-      <c r="Z22" s="169"/>
+      <c r="X22" s="159"/>
+      <c r="Y22" s="164"/>
+      <c r="Z22" s="162"/>
       <c r="AA22" s="12"/>
       <c r="AB22" s="12"/>
       <c r="AC22" s="13">
@@ -8904,7 +8892,7 @@
       </c>
     </row>
     <row r="23" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A23" s="128"/>
+      <c r="A23" s="120"/>
       <c r="W23" s="14"/>
       <c r="X23" s="16"/>
       <c r="Y23" s="37"/>
@@ -8923,26 +8911,26 @@
       </c>
     </row>
     <row r="24" spans="1:32" ht="15.5" x14ac:dyDescent="0.3">
-      <c r="A24" s="128"/>
-      <c r="B24" s="191"/>
-      <c r="C24" s="192"/>
-      <c r="D24" s="192"/>
-      <c r="E24" s="192"/>
-      <c r="F24" s="192"/>
-      <c r="G24" s="192"/>
-      <c r="H24" s="192"/>
-      <c r="I24" s="192"/>
-      <c r="J24" s="192"/>
-      <c r="K24" s="192"/>
-      <c r="L24" s="192"/>
-      <c r="M24" s="192"/>
-      <c r="N24" s="192"/>
-      <c r="O24" s="192"/>
-      <c r="P24" s="192"/>
-      <c r="Q24" s="192"/>
-      <c r="R24" s="192"/>
-      <c r="S24" s="192"/>
-      <c r="T24" s="193"/>
+      <c r="A24" s="120"/>
+      <c r="B24" s="137"/>
+      <c r="C24" s="138"/>
+      <c r="D24" s="138"/>
+      <c r="E24" s="138"/>
+      <c r="F24" s="138"/>
+      <c r="G24" s="138"/>
+      <c r="H24" s="138"/>
+      <c r="I24" s="138"/>
+      <c r="J24" s="138"/>
+      <c r="K24" s="138"/>
+      <c r="L24" s="138"/>
+      <c r="M24" s="138"/>
+      <c r="N24" s="138"/>
+      <c r="O24" s="138"/>
+      <c r="P24" s="138"/>
+      <c r="Q24" s="138"/>
+      <c r="R24" s="138"/>
+      <c r="S24" s="138"/>
+      <c r="T24" s="139"/>
       <c r="U24" s="15"/>
       <c r="V24" s="15">
         <f>SUM(V16:V22)</f>
@@ -8959,22 +8947,22 @@
       </c>
     </row>
     <row r="27" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="I27" s="119"/>
-      <c r="J27" s="119"/>
-      <c r="K27" s="119"/>
-      <c r="L27" s="119"/>
+      <c r="I27" s="117"/>
+      <c r="J27" s="117"/>
+      <c r="K27" s="117"/>
+      <c r="L27" s="117"/>
     </row>
     <row r="29" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="L29" s="119"/>
-      <c r="M29" s="119"/>
-      <c r="N29" s="119"/>
-      <c r="O29" s="119"/>
+      <c r="L29" s="117"/>
+      <c r="M29" s="117"/>
+      <c r="N29" s="117"/>
+      <c r="O29" s="117"/>
     </row>
     <row r="30" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="L30" s="119"/>
-      <c r="M30" s="119"/>
-      <c r="N30" s="119"/>
-      <c r="O30" s="119"/>
+      <c r="L30" s="117"/>
+      <c r="M30" s="117"/>
+      <c r="N30" s="117"/>
+      <c r="O30" s="117"/>
     </row>
     <row r="31" spans="1:32" x14ac:dyDescent="0.3">
       <c r="AF31" t="s">
@@ -8983,16 +8971,33 @@
     </row>
   </sheetData>
   <mergeCells count="53">
-    <mergeCell ref="L29:M29"/>
-    <mergeCell ref="N29:O29"/>
-    <mergeCell ref="L30:M30"/>
-    <mergeCell ref="N30:O30"/>
-    <mergeCell ref="Z16:Z22"/>
-    <mergeCell ref="K18:K22"/>
-    <mergeCell ref="Y18:Y22"/>
-    <mergeCell ref="B24:T24"/>
-    <mergeCell ref="I27:J27"/>
-    <mergeCell ref="K27:L27"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="V14:V15"/>
+    <mergeCell ref="S2:S3"/>
+    <mergeCell ref="T2:U3"/>
+    <mergeCell ref="A14:A24"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:M2"/>
+    <mergeCell ref="O2:O3"/>
+    <mergeCell ref="P2:P3"/>
+    <mergeCell ref="Q2:Q3"/>
+    <mergeCell ref="R2:R3"/>
+    <mergeCell ref="I14:I15"/>
+    <mergeCell ref="J14:J15"/>
+    <mergeCell ref="K14:K15"/>
+    <mergeCell ref="T14:T15"/>
+    <mergeCell ref="U14:U15"/>
     <mergeCell ref="AC14:AC15"/>
     <mergeCell ref="C16:C22"/>
     <mergeCell ref="E16:E22"/>
@@ -9009,33 +9014,16 @@
     <mergeCell ref="Z14:Z15"/>
     <mergeCell ref="AA14:AA15"/>
     <mergeCell ref="AB14:AB15"/>
-    <mergeCell ref="I14:I15"/>
-    <mergeCell ref="J14:J15"/>
-    <mergeCell ref="K14:K15"/>
-    <mergeCell ref="T14:T15"/>
-    <mergeCell ref="U14:U15"/>
-    <mergeCell ref="V14:V15"/>
-    <mergeCell ref="S2:S3"/>
-    <mergeCell ref="T2:U3"/>
-    <mergeCell ref="A14:A24"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="F14:F15"/>
-    <mergeCell ref="G14:G15"/>
-    <mergeCell ref="H14:H15"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:M2"/>
-    <mergeCell ref="O2:O3"/>
-    <mergeCell ref="P2:P3"/>
-    <mergeCell ref="Q2:Q3"/>
-    <mergeCell ref="R2:R3"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="A2:A4"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="K18:K22"/>
+    <mergeCell ref="Y18:Y22"/>
+    <mergeCell ref="B24:T24"/>
+    <mergeCell ref="I27:J27"/>
+    <mergeCell ref="K27:L27"/>
+    <mergeCell ref="L29:M29"/>
+    <mergeCell ref="N29:O29"/>
+    <mergeCell ref="L30:M30"/>
+    <mergeCell ref="N30:O30"/>
+    <mergeCell ref="Z16:Z22"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9068,7 +9056,7 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="128" t="s">
+      <c r="A2" s="120" t="s">
         <v>0</v>
       </c>
       <c r="B2" t="s">
@@ -9085,7 +9073,7 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="128"/>
+      <c r="A3" s="120"/>
       <c r="B3" t="s">
         <v>188</v>
       </c>
@@ -9100,7 +9088,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="128"/>
+      <c r="A4" s="120"/>
       <c r="B4" t="s">
         <v>188</v>
       </c>
@@ -9129,7 +9117,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="128" t="s">
+      <c r="A10" s="120" t="s">
         <v>0</v>
       </c>
       <c r="B10" t="s">
@@ -9146,7 +9134,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="128"/>
+      <c r="A11" s="120"/>
       <c r="B11" t="s">
         <v>188</v>
       </c>
@@ -9161,7 +9149,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="128"/>
+      <c r="A12" s="120"/>
       <c r="B12" t="s">
         <v>188</v>
       </c>
@@ -9190,7 +9178,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="128" t="s">
+      <c r="A17" s="120" t="s">
         <v>0</v>
       </c>
       <c r="B17" t="s">
@@ -9207,7 +9195,7 @@
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="128"/>
+      <c r="A18" s="120"/>
       <c r="B18" t="s">
         <v>188</v>
       </c>
@@ -9222,7 +9210,7 @@
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="128"/>
+      <c r="A19" s="120"/>
       <c r="B19" t="s">
         <v>188</v>
       </c>
@@ -9251,7 +9239,7 @@
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="128" t="s">
+      <c r="A23" s="120" t="s">
         <v>0</v>
       </c>
       <c r="B23" t="s">
@@ -9268,7 +9256,7 @@
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" s="128"/>
+      <c r="A24" s="120"/>
       <c r="B24" t="s">
         <v>188</v>
       </c>
@@ -9283,7 +9271,7 @@
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" s="128"/>
+      <c r="A25" s="120"/>
       <c r="B25" t="s">
         <v>188</v>
       </c>
@@ -9312,7 +9300,7 @@
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A28" s="128" t="s">
+      <c r="A28" s="120" t="s">
         <v>0</v>
       </c>
       <c r="B28" t="s">
@@ -9326,7 +9314,7 @@
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A29" s="128"/>
+      <c r="A29" s="120"/>
       <c r="B29" s="82" t="s">
         <v>188</v>
       </c>
@@ -9338,7 +9326,7 @@
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A30" s="128"/>
+      <c r="A30" s="120"/>
       <c r="B30" s="82" t="s">
         <v>188</v>
       </c>

</xml_diff>